<commit_message>
Completed exercise of classifying all BRs against our Administrative domains and captured all BRs in separate design considerations doc
</commit_message>
<xml_diff>
--- a/docs/project-management/02_Business_Requirements/Northwind-Outdoor-RTM-v1.0.xlsx
+++ b/docs/project-management/02_Business_Requirements/Northwind-Outdoor-RTM-v1.0.xlsx
@@ -8,17 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/docs/project-management/02_Business_Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="262" documentId="8_{170D4D7C-E242-4887-90C6-7A678B36976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{309A0387-D55D-4B4E-A611-398DC9D6328D}"/>
+  <xr:revisionPtr revIDLastSave="472" documentId="8_{170D4D7C-E242-4887-90C6-7A678B36976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5783A1C2-7965-49AB-ABD3-D35792B2B3D4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="2" activeTab="4" xr2:uid="{BD0B86D2-9AC1-421E-A95D-1B17A25780EE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
     <sheet name="RTM" sheetId="2" r:id="rId2"/>
     <sheet name="Legend &amp; Reference" sheetId="3" r:id="rId3"/>
     <sheet name="Architecture Domains" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1386" uniqueCount="504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="550">
   <si>
     <t>Northwind Outdoor Ltd. | RTM Summary</t>
   </si>
@@ -1381,45 +1379,15 @@
     <t>AD-01, AD-02,AD-05</t>
   </si>
   <si>
-    <t>Role</t>
-  </si>
-  <si>
-    <t>Domain</t>
-  </si>
-  <si>
-    <t>Primary</t>
-  </si>
-  <si>
-    <t>Key Supporting</t>
-  </si>
-  <si>
-    <t>Secondary</t>
-  </si>
-  <si>
-    <t>AD-05 Application &amp; Business Services</t>
-  </si>
-  <si>
     <t xml:space="preserve">AD-03, AD-05, AD-08, </t>
   </si>
   <si>
     <t>AD-11, AD-02, AD-09</t>
   </si>
   <si>
-    <t>AD-03 Identity &amp; Access Architecture</t>
-  </si>
-  <si>
-    <t>AD-08 Security Architecture</t>
-  </si>
-  <si>
     <t>AD-03, AD-05, AD-08</t>
   </si>
   <si>
-    <t>Why it relates</t>
-  </si>
-  <si>
-    <t>AD-09 Observability Architecture</t>
-  </si>
-  <si>
     <t>AD-08, AD-05, AD-10</t>
   </si>
   <si>
@@ -1438,9 +1406,6 @@
     <t>AD-06, AD-09, AD-07</t>
   </si>
   <si>
-    <t>AD-10 Management &amp; Operations Architecture</t>
-  </si>
-  <si>
     <t>AD-10, AD-05, AD-03</t>
   </si>
   <si>
@@ -1448,18 +1413,6 @@
   </si>
   <si>
     <t>AD-10, AD-06, AD-11, AD-02</t>
-  </si>
-  <si>
-    <t>AD-02 Compute &amp; Platform Architecture</t>
-  </si>
-  <si>
-    <t>AD-01 Network Architecture</t>
-  </si>
-  <si>
-    <t>AD-04 Core Infrastructure Services</t>
-  </si>
-  <si>
-    <t>AD-12 Resilience &amp; Availability Architecture</t>
   </si>
   <si>
     <t>AD-10, AD-08, AD-07</t>
@@ -1536,37 +1489,220 @@
     <t>AD-10, AD-05, AD-02, AD-11, AD-12</t>
   </si>
   <si>
-    <t>Logical separation of systems/services is fundamentally a network architecture capability. The network design determines the segmentation model, boundaries and permitted connectivity between segments.</t>
-  </si>
-  <si>
-    <t>Improved security is an explicit outcome. Segmentation should limit unnecessary access and reduce the ability of a compromised system to reach unrelated infrastructure.</t>
-  </si>
-  <si>
-    <t>Operational resilience is also explicit. Segmentation can contain failures, reduce blast radius and separate systems with different operational/security characteristics.</t>
-  </si>
-  <si>
-    <t>Workloads must be placed into appropriate logical network/security zones. The compute architecture therefore needs to support the segmentation model.</t>
-  </si>
-  <si>
-    <t>Service placement and legitimate application communication requirements determine which segments need to communicate.</t>
-  </si>
-  <si>
-    <t>Administrative access across segments, changes to segmentation policy and troubleshooting require controlled operational processes.</t>
-  </si>
-  <si>
-    <t>Cross-segment traffic, denied connections and segment health may need logging/monitoring.</t>
-  </si>
-  <si>
-    <t>Certain access decisions may involve user/admin roles, particularly management access, although segmentation itself is primarily network-based.</t>
-  </si>
-  <si>
-    <t>Shared DNS, DHCP, NTP and similar services may need to operate across multiple segments and therefore influence permitted network flows.</t>
-  </si>
-  <si>
     <t>AD-08, AD-12, AD-02</t>
   </si>
   <si>
     <t>AD-05, AD-10, AD-09, AD-03, AD-04</t>
+  </si>
+  <si>
+    <t>AD-05, AD-03, AD-01</t>
+  </si>
+  <si>
+    <t>AD-08, AD-10, AD-02, AD-09, AD-12</t>
+  </si>
+  <si>
+    <t>AD-12, AD-05, AD-06</t>
+  </si>
+  <si>
+    <t>AD-01, AD-04, AD-08, AD-10, AD-09, AD-07</t>
+  </si>
+  <si>
+    <t>AD-06, AD-01, AD-05</t>
+  </si>
+  <si>
+    <t>AD-03, AD-04, AD-09, AD-10, AD-08, AD-07, AD-12</t>
+  </si>
+  <si>
+    <t>AD-02, AD-08, AD-04</t>
+  </si>
+  <si>
+    <t>AD-01, AD-03, AD-05, AD-06, AD-09, AD-07, AD-12</t>
+  </si>
+  <si>
+    <t>AD-12, AD-07, AD-05</t>
+  </si>
+  <si>
+    <t>AD-02, AD-01, AD-03, AD-04, AD-06, AD-08, AD-09, AD-11</t>
+  </si>
+  <si>
+    <t>AD-10, AD-08, AD-06</t>
+  </si>
+  <si>
+    <t>AD-02, AD-05, AD-01, AD-07, AD-12, AD-03</t>
+  </si>
+  <si>
+    <t>AD-03, AD-08, AD-09</t>
+  </si>
+  <si>
+    <t>AD-05, AD-02, AD-11</t>
+  </si>
+  <si>
+    <t>AD-01, AD-03, AD-10</t>
+  </si>
+  <si>
+    <t>AD-02, AD-08, AD-09, AD-12</t>
+  </si>
+  <si>
+    <t>AD-02, AD-08, AD-09</t>
+  </si>
+  <si>
+    <t>AD-01, AD-05, AD-11</t>
+  </si>
+  <si>
+    <t>AD-08, AD-02, AD-12</t>
+  </si>
+  <si>
+    <t>AD-05, AD-09, AD-07, AD-11</t>
+  </si>
+  <si>
+    <t>AD-02, AD-08, AD-05</t>
+  </si>
+  <si>
+    <t>AD-09, AD-12, AD-11</t>
+  </si>
+  <si>
+    <t>AD-02, AD-03, AD-08</t>
+  </si>
+  <si>
+    <t>AD-05, AD-06, AD-09, AD-07, AD-04, AD-01</t>
+  </si>
+  <si>
+    <t>AD-07, AD-05, AD-06, AD-04, AD-12</t>
+  </si>
+  <si>
+    <t>AD-09, AD-02, AD-06</t>
+  </si>
+  <si>
+    <t>AD-01, AD-05, AD-07, AD-12, AD-04</t>
+  </si>
+  <si>
+    <t>AD-03, AD-09, AD-08</t>
+  </si>
+  <si>
+    <t>AD-10, AD-02, AD-01, AD-05</t>
+  </si>
+  <si>
+    <t>AD-03, AD-02, AD-10</t>
+  </si>
+  <si>
+    <t>AD-01, AD-05, AD-06, AD-09</t>
+  </si>
+  <si>
+    <t>AD-03, AD-08, AD-10</t>
+  </si>
+  <si>
+    <t>AD-05, AD-04, AD-02, AD-09, AD-12</t>
+  </si>
+  <si>
+    <t>AD-09, AD-02, AD-08</t>
+  </si>
+  <si>
+    <t>AD-01, AD-05, AD-03, AD-04, AD-06, AD-07, AD-12, AD-11</t>
+  </si>
+  <si>
+    <t>AD-07 Backup &amp; Recovery, AD-02 Compute &amp; Platform, AD-09 Observability</t>
+  </si>
+  <si>
+    <t>AD-01, AD-04, AD-05, AD-06, AD-10</t>
+  </si>
+  <si>
+    <t>AD-02 Compute &amp; Platform, AD-10 Management &amp; Operations, AD-09 Observability</t>
+  </si>
+  <si>
+    <t>AD-01, AD-04, AD-05, AD-06, AD-07, AD-08</t>
+  </si>
+  <si>
+    <t>AD-06 Storage, AD-09 Observability, AD-01 Network</t>
+  </si>
+  <si>
+    <t>AD-05, AD-10, AD-12</t>
+  </si>
+  <si>
+    <t>AD-06 Storage, AD-01 Network, AD-10 Management &amp; Operations</t>
+  </si>
+  <si>
+    <t>AD-03, AD-04, AD-05, AD-09, AD-12</t>
+  </si>
+  <si>
+    <t>AD-03 Identity &amp; Access, AD-01 Network, AD-10 Management &amp; Operations</t>
+  </si>
+  <si>
+    <t>AD-02, AD-05, AD-06, AD-09, AD-11</t>
+  </si>
+  <si>
+    <t>AD-08 Security, AD-10 Management &amp; Operations, AD-03 Identity &amp; Access</t>
+  </si>
+  <si>
+    <t>AD-02, AD-05, AD-11</t>
+  </si>
+  <si>
+    <t>AD-03 Identity &amp; Access, AD-07 Backup &amp; Recovery, AD-06 Storage</t>
+  </si>
+  <si>
+    <t>AD-05, AD-09, AD-10, AD-11</t>
+  </si>
+  <si>
+    <t>AD-02 Compute &amp; Platform, AD-24-equivalent standardisation via BR-024 / AD-08 Security, AD-09 Observability</t>
+  </si>
+  <si>
+    <t>AD-01, AD-04, AD-05, AD-06, AD-07</t>
+  </si>
+  <si>
+    <t>AD-12 Resilience &amp; Availability, AD-10 Management &amp; Operations, AD-02 Compute &amp; Platform</t>
+  </si>
+  <si>
+    <t>AD-05, AD-06, AD-09, AD-04, AD-03</t>
+  </si>
+  <si>
+    <t>AD-09 Observability, AD-02 Compute &amp; Platform, AD-12 Resilience &amp; Availability</t>
+  </si>
+  <si>
+    <t>AD-05, AD-07, AD-08, AD-03, AD-04</t>
+  </si>
+  <si>
+    <t>AD-02 Compute &amp; Platform, AD-03 Identity &amp; Access, AD-08 Security</t>
+  </si>
+  <si>
+    <t>AD-04, AD-05, AD-09, AD-01</t>
+  </si>
+  <si>
+    <t>AD-05 Application &amp; Business Services, AD-03 Identity &amp; Access, AD-01 Network</t>
+  </si>
+  <si>
+    <t>AD-02, AD-08, AD-10, AD-04</t>
+  </si>
+  <si>
+    <t>AD-10 Management &amp; Operations, AD-09 Observability, AD-03 Identity &amp; Access</t>
+  </si>
+  <si>
+    <t>AD-05, AD-06, AD-07, AD-11</t>
+  </si>
+  <si>
+    <t>AD-10 Management &amp; Operations, AD-08 Security, AD-02 Compute &amp; Platform</t>
+  </si>
+  <si>
+    <t>AD-01, AD-04, AD-05, AD-06, AD-07, AD-12</t>
+  </si>
+  <si>
+    <t>AD-01 Network, AD-10 Management &amp; Operations, AD-11 Integration</t>
+  </si>
+  <si>
+    <t>AD-03, AD-04, AD-05, AD-06, AD-08, AD-09, AD-12</t>
+  </si>
+  <si>
+    <t>AD-02 Compute &amp; Platform, AD-08 Security, AD-09 Observability</t>
+  </si>
+  <si>
+    <t>AD-01, AD-03, AD-04, AD-05, AD-06, AD-07</t>
+  </si>
+  <si>
+    <t>AD-07 Backup &amp; Recovery, AD-10 Management &amp; Operations, AD-02 Compute &amp; Platform</t>
+  </si>
+  <si>
+    <t>AD-05, AD-06, AD-09, AD-08</t>
+  </si>
+  <si>
+    <t>AD-03 Identity &amp; Access, AD-09 Observability, AD-08 Security</t>
   </si>
 </sst>
 </file>
@@ -2945,21 +3081,24 @@
   <dimension ref="A1:W60"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="1" max="1" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="12" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="11" customWidth="1"/>
-    <col min="9" max="9" width="12" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="13" width="17" customWidth="1"/>
-    <col min="14" max="14" width="15.25" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="17" customWidth="1"/>
+    <col min="5" max="5" width="6.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="16" max="19" width="11.5" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="42" customWidth="1"/>
-    <col min="21" max="21" width="22" customWidth="1"/>
-    <col min="22" max="22" width="26" customWidth="1"/>
+    <col min="21" max="21" width="19.625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="25" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="54" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3269,10 +3408,10 @@
         <v>428</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="P7" s="4" t="s">
         <v>57</v>
@@ -3340,10 +3479,10 @@
         <v>428</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="P8" s="4" t="s">
         <v>57</v>
@@ -3411,10 +3550,10 @@
         <v>400</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>460</v>
+        <v>450</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>461</v>
+        <v>451</v>
       </c>
       <c r="P9" s="4" t="s">
         <v>57</v>
@@ -3482,10 +3621,10 @@
         <v>408</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>462</v>
+        <v>452</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>463</v>
+        <v>453</v>
       </c>
       <c r="P10" s="4" t="s">
         <v>57</v>
@@ -3553,10 +3692,10 @@
         <v>408</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>464</v>
+        <v>454</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>465</v>
+        <v>455</v>
       </c>
       <c r="P11" s="4" t="s">
         <v>57</v>
@@ -3624,10 +3763,10 @@
         <v>420</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>467</v>
+        <v>456</v>
       </c>
       <c r="O12" s="4" t="s">
-        <v>465</v>
+        <v>455</v>
       </c>
       <c r="P12" s="4" t="s">
         <v>57</v>
@@ -3695,10 +3834,10 @@
         <v>420</v>
       </c>
       <c r="N13" s="4" t="s">
-        <v>468</v>
+        <v>457</v>
       </c>
       <c r="O13" s="4" t="s">
-        <v>469</v>
+        <v>458</v>
       </c>
       <c r="P13" s="4" t="s">
         <v>57</v>
@@ -3837,10 +3976,10 @@
         <v>424</v>
       </c>
       <c r="N15" s="4" t="s">
-        <v>474</v>
+        <v>459</v>
       </c>
       <c r="O15" s="4" t="s">
-        <v>475</v>
+        <v>460</v>
       </c>
       <c r="P15" s="4" t="s">
         <v>57</v>
@@ -3908,10 +4047,10 @@
         <v>420</v>
       </c>
       <c r="N16" s="4" t="s">
-        <v>476</v>
+        <v>461</v>
       </c>
       <c r="O16" s="4" t="s">
-        <v>477</v>
+        <v>462</v>
       </c>
       <c r="P16" s="4" t="s">
         <v>57</v>
@@ -3979,10 +4118,10 @@
         <v>416</v>
       </c>
       <c r="N17" s="4" t="s">
-        <v>478</v>
+        <v>463</v>
       </c>
       <c r="O17" s="4" t="s">
-        <v>479</v>
+        <v>464</v>
       </c>
       <c r="P17" s="4" t="s">
         <v>57</v>
@@ -4050,10 +4189,10 @@
         <v>416</v>
       </c>
       <c r="N18" s="4" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="O18" s="4" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="P18" s="4" t="s">
         <v>57</v>
@@ -4121,10 +4260,10 @@
         <v>436</v>
       </c>
       <c r="N19" s="4" t="s">
-        <v>482</v>
+        <v>467</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>483</v>
+        <v>468</v>
       </c>
       <c r="P19" s="4" t="s">
         <v>57</v>
@@ -4162,7 +4301,7 @@
         <v>23</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>486</v>
+        <v>471</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>24</v>
@@ -4192,10 +4331,10 @@
         <v>436</v>
       </c>
       <c r="N20" s="4" t="s">
-        <v>484</v>
+        <v>469</v>
       </c>
       <c r="O20" s="4" t="s">
-        <v>485</v>
+        <v>470</v>
       </c>
       <c r="P20" s="4" t="s">
         <v>57</v>
@@ -4263,10 +4402,10 @@
         <v>428</v>
       </c>
       <c r="N21" s="4" t="s">
-        <v>487</v>
+        <v>472</v>
       </c>
       <c r="O21" s="4" t="s">
-        <v>488</v>
+        <v>473</v>
       </c>
       <c r="P21" s="4" t="s">
         <v>57</v>
@@ -4334,10 +4473,10 @@
         <v>392</v>
       </c>
       <c r="N22" s="4" t="s">
-        <v>489</v>
+        <v>474</v>
       </c>
       <c r="O22" s="4" t="s">
-        <v>490</v>
+        <v>475</v>
       </c>
       <c r="P22" s="4" t="s">
         <v>57</v>
@@ -4405,10 +4544,10 @@
         <v>420</v>
       </c>
       <c r="N23" s="4" t="s">
-        <v>491</v>
+        <v>476</v>
       </c>
       <c r="O23" s="4" t="s">
-        <v>492</v>
+        <v>477</v>
       </c>
       <c r="P23" s="4" t="s">
         <v>57</v>
@@ -4476,10 +4615,10 @@
         <v>392</v>
       </c>
       <c r="N24" s="4" t="s">
-        <v>502</v>
+        <v>478</v>
       </c>
       <c r="O24" s="4" t="s">
-        <v>503</v>
+        <v>479</v>
       </c>
       <c r="P24" s="4" t="s">
         <v>57</v>
@@ -4543,9 +4682,15 @@
       <c r="L25" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M25" s="4"/>
-      <c r="N25" s="4"/>
-      <c r="O25" s="4"/>
+      <c r="M25" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="N25" s="4" t="s">
+        <v>480</v>
+      </c>
+      <c r="O25" s="4" t="s">
+        <v>481</v>
+      </c>
       <c r="P25" s="4" t="s">
         <v>57</v>
       </c>
@@ -4608,9 +4753,15 @@
       <c r="L26" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M26" s="4"/>
-      <c r="N26" s="4"/>
-      <c r="O26" s="4"/>
+      <c r="M26" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="N26" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="O26" s="4" t="s">
+        <v>483</v>
+      </c>
       <c r="P26" s="4" t="s">
         <v>57</v>
       </c>
@@ -4673,9 +4824,15 @@
       <c r="L27" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M27" s="4"/>
-      <c r="N27" s="4"/>
-      <c r="O27" s="4"/>
+      <c r="M27" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="N27" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="O27" s="4" t="s">
+        <v>485</v>
+      </c>
       <c r="P27" s="4" t="s">
         <v>57</v>
       </c>
@@ -4738,9 +4895,15 @@
       <c r="L28" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M28" s="4"/>
-      <c r="N28" s="4"/>
-      <c r="O28" s="4"/>
+      <c r="M28" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N28" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="O28" s="4" t="s">
+        <v>487</v>
+      </c>
       <c r="P28" s="4" t="s">
         <v>57</v>
       </c>
@@ -4803,9 +4966,15 @@
       <c r="L29" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M29" s="4"/>
-      <c r="N29" s="4"/>
-      <c r="O29" s="4"/>
+      <c r="M29" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N29" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="O29" s="4" t="s">
+        <v>489</v>
+      </c>
       <c r="P29" s="4" t="s">
         <v>57</v>
       </c>
@@ -4868,9 +5037,15 @@
       <c r="L30" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M30" s="4"/>
-      <c r="N30" s="4"/>
-      <c r="O30" s="4"/>
+      <c r="M30" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="N30" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="O30" s="4" t="s">
+        <v>491</v>
+      </c>
       <c r="P30" s="4" t="s">
         <v>57</v>
       </c>
@@ -4933,9 +5108,15 @@
       <c r="L31" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M31" s="4"/>
-      <c r="N31" s="4"/>
-      <c r="O31" s="4"/>
+      <c r="M31" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N31" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="O31" s="4" t="s">
+        <v>493</v>
+      </c>
       <c r="P31" s="4" t="s">
         <v>57</v>
       </c>
@@ -4998,9 +5179,15 @@
       <c r="L32" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M32" s="4"/>
-      <c r="N32" s="4"/>
-      <c r="O32" s="4"/>
+      <c r="M32" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="N32" s="4" t="s">
+        <v>494</v>
+      </c>
+      <c r="O32" s="4" t="s">
+        <v>495</v>
+      </c>
       <c r="P32" s="4" t="s">
         <v>57</v>
       </c>
@@ -5063,9 +5250,15 @@
       <c r="L33" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M33" s="4"/>
-      <c r="N33" s="4"/>
-      <c r="O33" s="4"/>
+      <c r="M33" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N33" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="O33" s="4" t="s">
+        <v>497</v>
+      </c>
       <c r="P33" s="4" t="s">
         <v>57</v>
       </c>
@@ -5128,9 +5321,15 @@
       <c r="L34" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M34" s="4"/>
-      <c r="N34" s="4"/>
-      <c r="O34" s="4"/>
+      <c r="M34" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N34" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="O34" s="4" t="s">
+        <v>499</v>
+      </c>
       <c r="P34" s="4" t="s">
         <v>57</v>
       </c>
@@ -5193,9 +5392,15 @@
       <c r="L35" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M35" s="4"/>
-      <c r="N35" s="4"/>
-      <c r="O35" s="4"/>
+      <c r="M35" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N35" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="O35" s="4" t="s">
+        <v>501</v>
+      </c>
       <c r="P35" s="4" t="s">
         <v>57</v>
       </c>
@@ -5258,9 +5463,15 @@
       <c r="L36" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M36" s="4"/>
-      <c r="N36" s="4"/>
-      <c r="O36" s="4"/>
+      <c r="M36" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N36" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="O36" s="4" t="s">
+        <v>503</v>
+      </c>
       <c r="P36" s="4" t="s">
         <v>57</v>
       </c>
@@ -5323,9 +5534,15 @@
       <c r="L37" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M37" s="4"/>
-      <c r="N37" s="4"/>
-      <c r="O37" s="4"/>
+      <c r="M37" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N37" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="O37" s="4" t="s">
+        <v>504</v>
+      </c>
       <c r="P37" s="4" t="s">
         <v>57</v>
       </c>
@@ -5388,9 +5605,15 @@
       <c r="L38" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M38" s="4"/>
-      <c r="N38" s="4"/>
-      <c r="O38" s="4"/>
+      <c r="M38" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N38" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="O38" s="4" t="s">
+        <v>506</v>
+      </c>
       <c r="P38" s="4" t="s">
         <v>57</v>
       </c>
@@ -5453,9 +5676,15 @@
       <c r="L39" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M39" s="4"/>
-      <c r="N39" s="4"/>
-      <c r="O39" s="4"/>
+      <c r="M39" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="N39" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="O39" s="4" t="s">
+        <v>508</v>
+      </c>
       <c r="P39" s="4" t="s">
         <v>57</v>
       </c>
@@ -5518,9 +5747,15 @@
       <c r="L40" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M40" s="4"/>
-      <c r="N40" s="4"/>
-      <c r="O40" s="4"/>
+      <c r="M40" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="N40" s="4" t="s">
+        <v>509</v>
+      </c>
+      <c r="O40" s="4" t="s">
+        <v>510</v>
+      </c>
       <c r="P40" s="4" t="s">
         <v>57</v>
       </c>
@@ -5583,9 +5818,15 @@
       <c r="L41" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M41" s="4"/>
-      <c r="N41" s="4"/>
-      <c r="O41" s="4"/>
+      <c r="M41" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="N41" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="O41" s="4" t="s">
+        <v>512</v>
+      </c>
       <c r="P41" s="4" t="s">
         <v>57</v>
       </c>
@@ -5648,9 +5889,15 @@
       <c r="L42" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M42" s="4"/>
-      <c r="N42" s="4"/>
-      <c r="O42" s="4"/>
+      <c r="M42" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N42" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="O42" s="4" t="s">
+        <v>514</v>
+      </c>
       <c r="P42" s="4" t="s">
         <v>57</v>
       </c>
@@ -5713,9 +5960,15 @@
       <c r="L43" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M43" s="4"/>
-      <c r="N43" s="4"/>
-      <c r="O43" s="4"/>
+      <c r="M43" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="N43" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="O43" s="4" t="s">
+        <v>516</v>
+      </c>
       <c r="P43" s="4" t="s">
         <v>57</v>
       </c>
@@ -5778,9 +6031,15 @@
       <c r="L44" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M44" s="4"/>
-      <c r="N44" s="4"/>
-      <c r="O44" s="4"/>
+      <c r="M44" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="N44" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="O44" s="4" t="s">
+        <v>518</v>
+      </c>
       <c r="P44" s="4" t="s">
         <v>57</v>
       </c>
@@ -5843,9 +6102,15 @@
       <c r="L45" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M45" s="4"/>
-      <c r="N45" s="4"/>
-      <c r="O45" s="4"/>
+      <c r="M45" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="N45" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="O45" s="4" t="s">
+        <v>520</v>
+      </c>
       <c r="P45" s="4" t="s">
         <v>57</v>
       </c>
@@ -5908,9 +6173,15 @@
       <c r="L46" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M46" s="4"/>
-      <c r="N46" s="4"/>
-      <c r="O46" s="4"/>
+      <c r="M46" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="N46" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="O46" s="4" t="s">
+        <v>522</v>
+      </c>
       <c r="P46" s="4" t="s">
         <v>57</v>
       </c>
@@ -5973,9 +6244,15 @@
       <c r="L47" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M47" s="4"/>
-      <c r="N47" s="4"/>
-      <c r="O47" s="4"/>
+      <c r="M47" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="N47" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="O47" s="4" t="s">
+        <v>524</v>
+      </c>
       <c r="P47" s="4" t="s">
         <v>57</v>
       </c>
@@ -6038,9 +6315,15 @@
       <c r="L48" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M48" s="4"/>
-      <c r="N48" s="4"/>
-      <c r="O48" s="4"/>
+      <c r="M48" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="N48" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="O48" s="4" t="s">
+        <v>526</v>
+      </c>
       <c r="P48" s="4" t="s">
         <v>57</v>
       </c>
@@ -6103,9 +6386,15 @@
       <c r="L49" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M49" s="4"/>
-      <c r="N49" s="4"/>
-      <c r="O49" s="4"/>
+      <c r="M49" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="N49" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="O49" s="4" t="s">
+        <v>528</v>
+      </c>
       <c r="P49" s="4" t="s">
         <v>57</v>
       </c>
@@ -6168,9 +6457,15 @@
       <c r="L50" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M50" s="4"/>
-      <c r="N50" s="4"/>
-      <c r="O50" s="4"/>
+      <c r="M50" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N50" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="O50" s="4" t="s">
+        <v>530</v>
+      </c>
       <c r="P50" s="4" t="s">
         <v>57</v>
       </c>
@@ -6233,9 +6528,15 @@
       <c r="L51" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M51" s="4"/>
-      <c r="N51" s="4"/>
-      <c r="O51" s="4"/>
+      <c r="M51" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="N51" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="O51" s="4" t="s">
+        <v>532</v>
+      </c>
       <c r="P51" s="4" t="s">
         <v>57</v>
       </c>
@@ -6298,9 +6599,15 @@
       <c r="L52" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M52" s="4"/>
-      <c r="N52" s="4"/>
-      <c r="O52" s="4"/>
+      <c r="M52" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N52" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="O52" s="4" t="s">
+        <v>534</v>
+      </c>
       <c r="P52" s="4" t="s">
         <v>57</v>
       </c>
@@ -6363,9 +6670,15 @@
       <c r="L53" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M53" s="4"/>
-      <c r="N53" s="4"/>
-      <c r="O53" s="4"/>
+      <c r="M53" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N53" s="4" t="s">
+        <v>535</v>
+      </c>
+      <c r="O53" s="4" t="s">
+        <v>536</v>
+      </c>
       <c r="P53" s="4" t="s">
         <v>57</v>
       </c>
@@ -6428,9 +6741,15 @@
       <c r="L54" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M54" s="4"/>
-      <c r="N54" s="4"/>
-      <c r="O54" s="4"/>
+      <c r="M54" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="N54" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="O54" s="4" t="s">
+        <v>538</v>
+      </c>
       <c r="P54" s="4" t="s">
         <v>57</v>
       </c>
@@ -6493,9 +6812,15 @@
       <c r="L55" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M55" s="4"/>
-      <c r="N55" s="4"/>
-      <c r="O55" s="4"/>
+      <c r="M55" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="N55" s="4" t="s">
+        <v>539</v>
+      </c>
+      <c r="O55" s="4" t="s">
+        <v>540</v>
+      </c>
       <c r="P55" s="4" t="s">
         <v>57</v>
       </c>
@@ -6558,9 +6883,15 @@
       <c r="L56" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M56" s="4"/>
-      <c r="N56" s="4"/>
-      <c r="O56" s="4"/>
+      <c r="M56" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="N56" s="4" t="s">
+        <v>541</v>
+      </c>
+      <c r="O56" s="4" t="s">
+        <v>542</v>
+      </c>
       <c r="P56" s="4" t="s">
         <v>57</v>
       </c>
@@ -6623,9 +6954,15 @@
       <c r="L57" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M57" s="4"/>
-      <c r="N57" s="4"/>
-      <c r="O57" s="4"/>
+      <c r="M57" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="N57" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="O57" s="4" t="s">
+        <v>544</v>
+      </c>
       <c r="P57" s="4" t="s">
         <v>57</v>
       </c>
@@ -6688,9 +7025,15 @@
       <c r="L58" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M58" s="4"/>
-      <c r="N58" s="4"/>
-      <c r="O58" s="4"/>
+      <c r="M58" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="N58" s="4" t="s">
+        <v>545</v>
+      </c>
+      <c r="O58" s="4" t="s">
+        <v>546</v>
+      </c>
       <c r="P58" s="4" t="s">
         <v>57</v>
       </c>
@@ -6753,9 +7096,15 @@
       <c r="L59" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M59" s="4"/>
-      <c r="N59" s="4"/>
-      <c r="O59" s="4"/>
+      <c r="M59" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="N59" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="O59" s="4" t="s">
+        <v>548</v>
+      </c>
       <c r="P59" s="4" t="s">
         <v>57</v>
       </c>
@@ -6818,9 +7167,15 @@
       <c r="L60" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="M60" s="6"/>
-      <c r="N60" s="6"/>
-      <c r="O60" s="6"/>
+      <c r="M60" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="N60" s="6" t="s">
+        <v>549</v>
+      </c>
+      <c r="O60" s="6" t="s">
+        <v>508</v>
+      </c>
       <c r="P60" s="6" t="s">
         <v>57</v>
       </c>
@@ -7328,129 +7683,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE6F4BC9-6BA0-49D2-B9EC-3326267B383F}">
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultColWidth="27.125" defaultRowHeight="14.25"/>
-  <cols>
-    <col min="1" max="1" width="14.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="67.125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="15">
-      <c r="A1" s="40" t="s">
-        <v>447</v>
-      </c>
-      <c r="B1" s="40" t="s">
-        <v>448</v>
-      </c>
-      <c r="C1" s="40" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="57">
-      <c r="A2" s="42" t="s">
-        <v>449</v>
-      </c>
-      <c r="B2" s="42" t="s">
-        <v>471</v>
-      </c>
-      <c r="C2" s="41" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="42.75">
-      <c r="A3" s="42" t="s">
-        <v>450</v>
-      </c>
-      <c r="B3" s="42" t="s">
-        <v>456</v>
-      </c>
-      <c r="C3" s="41" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="42.75">
-      <c r="A4" s="42" t="s">
-        <v>450</v>
-      </c>
-      <c r="B4" s="42" t="s">
-        <v>473</v>
-      </c>
-      <c r="C4" s="41" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="42.75">
-      <c r="A5" s="42" t="s">
-        <v>450</v>
-      </c>
-      <c r="B5" s="42" t="s">
-        <v>470</v>
-      </c>
-      <c r="C5" s="41" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="30">
-      <c r="A6" s="42" t="s">
-        <v>451</v>
-      </c>
-      <c r="B6" s="42" t="s">
-        <v>452</v>
-      </c>
-      <c r="C6" s="41" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="30">
-      <c r="A7" s="42" t="s">
-        <v>451</v>
-      </c>
-      <c r="B7" s="42" t="s">
-        <v>466</v>
-      </c>
-      <c r="C7" s="41" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="30">
-      <c r="A8" s="42" t="s">
-        <v>451</v>
-      </c>
-      <c r="B8" s="42" t="s">
-        <v>459</v>
-      </c>
-      <c r="C8" s="41" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="42.75">
-      <c r="A9" s="42" t="s">
-        <v>451</v>
-      </c>
-      <c r="B9" s="42" t="s">
-        <v>455</v>
-      </c>
-      <c r="C9" s="41" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="42.75">
-      <c r="A10" s="42" t="s">
-        <v>451</v>
-      </c>
-      <c r="B10" s="42" t="s">
-        <v>472</v>
-      </c>
-      <c r="C10" s="41" t="s">
-        <v>501</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Created the HLD Design doc v0.1 to send to client. Completed the DD to BR mappings and refactored some HLD diagrams
</commit_message>
<xml_diff>
--- a/docs/project-management/02_Business_Requirements/Northwind-Outdoor-RTM-v1.0.xlsx
+++ b/docs/project-management/02_Business_Requirements/Northwind-Outdoor-RTM-v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/docs/project-management/02_Business_Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="642" documentId="8_{170D4D7C-E242-4887-90C6-7A678B36976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72A7FA09-7FC3-42C1-8F8F-356E6C972604}"/>
+  <xr:revisionPtr revIDLastSave="740" documentId="8_{170D4D7C-E242-4887-90C6-7A678B36976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D54EF7AD-19F9-4EF6-9BB7-D46AC06A5B15}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1476" uniqueCount="635">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1509" uniqueCount="663">
   <si>
     <t>Northwind Outdoor Ltd. | RTM Summary</t>
   </si>
@@ -1970,6 +1970,96 @@
   <si>
     <t>DD-002 — Identity &amp; Access Management Architecture
 DD-009 — Network Security &amp; Segmentation</t>
+  </si>
+  <si>
+    <t>DD-011 — Service Integration / Interoperability Architecture</t>
+  </si>
+  <si>
+    <t>DD-010 — Application Hosting Architecture</t>
+  </si>
+  <si>
+    <t>DD-001 — Compute / Platform Architecture</t>
+  </si>
+  <si>
+    <t>DD-001 — Compute / Platform Architecture
+DD-012 — Availability &amp; Resilience Strategy</t>
+  </si>
+  <si>
+    <t>DD-001 — Compute &amp; Platform Architecture</t>
+  </si>
+  <si>
+    <t>DD-004 — Storage Architecture
+DD-009 — Network Security &amp; Segmentation
+DD-012 — Availability &amp; Resilience Strategy</t>
+  </si>
+  <si>
+    <t>DD-011 — Automation &amp; Scheduled Operations Architecture</t>
+  </si>
+  <si>
+    <t>DD-010 — Application Hosting Architecture
+DD-012 — Availability &amp; Resilience Strategy</t>
+  </si>
+  <si>
+    <t>DD-006 — Monitoring &amp; Alerting</t>
+  </si>
+  <si>
+    <t>DD-007 — Logging &amp; Audit</t>
+  </si>
+  <si>
+    <t>No dedicated</t>
+  </si>
+  <si>
+    <t>DD-009 — Network Security &amp; Segmentation</t>
+  </si>
+  <si>
+    <t>DD-010 — Patch &amp; Software Lifecycle Management Architecture</t>
+  </si>
+  <si>
+    <t>DD-009 — Network Security &amp; Segmentation Architecture</t>
+  </si>
+  <si>
+    <t>DD-002 — Identity &amp; Access Management Architecture
+DD-008 — Remote Administration Architecture</t>
+  </si>
+  <si>
+    <t>DD-007 — Logging &amp; Audit
+DD-010 — Application Hosting Architecture</t>
+  </si>
+  <si>
+    <t>DD-005 — Backup &amp; Recovery Architecture; DD-006 — Monitoring &amp; Alerting Architecture</t>
+  </si>
+  <si>
+    <t>DD-001 — Compute / Virtualisation</t>
+  </si>
+  <si>
+    <t>DD-001 — Compute / Virtualisation; DD-004 — Storage Architecture</t>
+  </si>
+  <si>
+    <t>DD-004 — Storage Architecture; DD-012 — Availability &amp; Resilience Strategy</t>
+  </si>
+  <si>
+    <t>DD-002 — Identity &amp; Access Management Architecture; DD-008 — Remote &amp; Administrative Access Architecture</t>
+  </si>
+  <si>
+    <t>DD-002 — Identity &amp; Access Management Architecture; DD-005 — Backup &amp; Recovery Architecture</t>
+  </si>
+  <si>
+    <t>DD-010 — Patch &amp; Software Lifecycle Management Architecture; DD-001 — Compute / Virtualisation</t>
+  </si>
+  <si>
+    <t>DD-010 — Patch &amp; Software Lifecycle Management Architecture; DD-012 — Availability &amp; Resilience Strategy</t>
+  </si>
+  <si>
+    <t>DD-001 — Compute / Virtualisation; DD-008 — Remote &amp; Administrative Access Architecture</t>
+  </si>
+  <si>
+    <t>DD-007 — Logging &amp; Audit Architecture; DD-010 — Patch &amp; Software Lifecycle Management Architecture</t>
+  </si>
+  <si>
+    <t>DD-001 — Compute / Virtualisation; DD-010 — Patch &amp; Software Lifecycle Management Architecture</t>
+  </si>
+  <si>
+    <t>DD-005 — Backup &amp; Recovery Architecture; DD-010 — Patch &amp; Software Lifecycle Management Architecture</t>
   </si>
 </sst>
 </file>
@@ -2527,6 +2617,13 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2542,18 +2639,49 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="12">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -2587,23 +2715,6 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -3041,17 +3152,17 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="DF"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="BD"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="CAP (Primary)"/>
-    <tableColumn id="23" xr3:uid="{C116EC89-8261-41A9-893A-12DFD9AC01D5}" name="CAP (Secondary)" dataDxfId="5"/>
+    <tableColumn id="23" xr3:uid="{C116EC89-8261-41A9-893A-12DFD9AC01D5}" name="CAP (Secondary)" dataDxfId="11"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="BRD"/>
-    <tableColumn id="20" xr3:uid="{D1E0B300-86BD-45A9-B3EB-8951F17E8029}" name="Primary AD" dataDxfId="8"/>
-    <tableColumn id="22" xr3:uid="{701B3B8E-55FF-4520-83AD-295760593E66}" name="Key ADs" dataDxfId="7"/>
-    <tableColumn id="21" xr3:uid="{1638868F-A11C-40F1-8FB2-2AB197E42B79}" name="Secondary Ads" dataDxfId="6"/>
+    <tableColumn id="20" xr3:uid="{D1E0B300-86BD-45A9-B3EB-8951F17E8029}" name="Primary AD" dataDxfId="10"/>
+    <tableColumn id="22" xr3:uid="{701B3B8E-55FF-4520-83AD-295760593E66}" name="Key ADs" dataDxfId="9"/>
+    <tableColumn id="21" xr3:uid="{1638868F-A11C-40F1-8FB2-2AB197E42B79}" name="Secondary Ads" dataDxfId="8"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="HLD (Primary)"/>
-    <tableColumn id="24" xr3:uid="{599BD185-8391-4930-BB9A-B52E39596ACD}" name="HLD (Secondary)" dataDxfId="4"/>
+    <tableColumn id="24" xr3:uid="{599BD185-8391-4930-BB9A-B52E39596ACD}" name="HLD (Secondary)" dataDxfId="7"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="LLD"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="ADR"/>
-    <tableColumn id="25" xr3:uid="{28378BB4-B208-482C-96C2-5A1994DECC42}" name="SOW" dataDxfId="3"/>
-    <tableColumn id="26" xr3:uid="{BAEC8EC4-D90B-4FBA-979D-21CDBE3C330A}" name="Sprint" dataDxfId="0"/>
+    <tableColumn id="25" xr3:uid="{28378BB4-B208-482C-96C2-5A1994DECC42}" name="SOW" dataDxfId="6"/>
+    <tableColumn id="26" xr3:uid="{BAEC8EC4-D90B-4FBA-979D-21CDBE3C330A}" name="Sprint" dataDxfId="5"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Test / UAT"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Acceptance Criteria"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Status"/>
@@ -3272,32 +3383,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="27.95" customHeight="1">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
     </row>
     <row r="2" spans="1:10" ht="21" customHeight="1">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
     </row>
     <row r="4" spans="1:10" ht="15">
       <c r="A4" s="21" t="s">
@@ -3501,7 +3612,7 @@
     <col min="13" max="13" width="19.875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15.625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16" customWidth="1"/>
+    <col min="16" max="16" width="26.375" customWidth="1"/>
     <col min="17" max="18" width="11.5" bestFit="1" customWidth="1"/>
     <col min="19" max="20" width="11.5" customWidth="1"/>
     <col min="21" max="21" width="11.5" bestFit="1" customWidth="1"/>
@@ -3512,60 +3623,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="27.95" customHeight="1">
-      <c r="B1" s="43" t="s">
+      <c r="B1" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="43"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="43"/>
-      <c r="T1" s="43"/>
-      <c r="U1" s="43"/>
-      <c r="V1" s="43"/>
-      <c r="W1" s="43"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="43"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
+      <c r="P1" s="46"/>
+      <c r="Q1" s="46"/>
+      <c r="R1" s="46"/>
+      <c r="S1" s="46"/>
+      <c r="T1" s="46"/>
+      <c r="U1" s="46"/>
+      <c r="V1" s="46"/>
+      <c r="W1" s="46"/>
+      <c r="X1" s="46"/>
+      <c r="Y1" s="46"/>
     </row>
     <row r="2" spans="1:25" ht="21" customHeight="1">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="44"/>
-      <c r="L2" s="44"/>
-      <c r="M2" s="44"/>
-      <c r="N2" s="44"/>
-      <c r="O2" s="44"/>
-      <c r="P2" s="44"/>
-      <c r="Q2" s="44"/>
-      <c r="R2" s="44"/>
-      <c r="S2" s="44"/>
-      <c r="T2" s="44"/>
-      <c r="U2" s="44"/>
-      <c r="V2" s="44"/>
-      <c r="W2" s="44"/>
-      <c r="X2" s="44"/>
-      <c r="Y2" s="44"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
+      <c r="P2" s="47"/>
+      <c r="Q2" s="47"/>
+      <c r="R2" s="47"/>
+      <c r="S2" s="47"/>
+      <c r="T2" s="47"/>
+      <c r="U2" s="47"/>
+      <c r="V2" s="47"/>
+      <c r="W2" s="47"/>
+      <c r="X2" s="47"/>
+      <c r="Y2" s="47"/>
     </row>
     <row r="4" spans="1:25" ht="33" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -4903,9 +5014,11 @@
         <v>475</v>
       </c>
       <c r="O22" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P22" s="4"/>
+        <v>633</v>
+      </c>
+      <c r="P22" s="4" t="s">
+        <v>634</v>
+      </c>
       <c r="Q22" s="4" t="s">
         <v>57</v>
       </c>
@@ -4974,9 +5087,11 @@
         <v>477</v>
       </c>
       <c r="O23" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P23" s="4"/>
+        <v>626</v>
+      </c>
+      <c r="P23" s="4" t="s">
+        <v>621</v>
+      </c>
       <c r="Q23" s="4" t="s">
         <v>57</v>
       </c>
@@ -5045,9 +5160,11 @@
         <v>479</v>
       </c>
       <c r="O24" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P24" s="4"/>
+        <v>626</v>
+      </c>
+      <c r="P24" s="4" t="s">
+        <v>637</v>
+      </c>
       <c r="Q24" s="4" t="s">
         <v>57</v>
       </c>
@@ -5114,7 +5231,7 @@
         <v>481</v>
       </c>
       <c r="O25" s="4" t="s">
-        <v>57</v>
+        <v>635</v>
       </c>
       <c r="P25" s="4"/>
       <c r="Q25" s="4" t="s">
@@ -5185,9 +5302,11 @@
         <v>483</v>
       </c>
       <c r="O26" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P26" s="4"/>
+        <v>636</v>
+      </c>
+      <c r="P26" s="4" t="s">
+        <v>638</v>
+      </c>
       <c r="Q26" s="4" t="s">
         <v>57</v>
       </c>
@@ -5254,9 +5373,11 @@
         <v>485</v>
       </c>
       <c r="O27" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P27" s="4"/>
+        <v>639</v>
+      </c>
+      <c r="P27" s="4" t="s">
+        <v>640</v>
+      </c>
       <c r="Q27" s="4" t="s">
         <v>57</v>
       </c>
@@ -5325,9 +5446,11 @@
         <v>487</v>
       </c>
       <c r="O28" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P28" s="4"/>
+        <v>637</v>
+      </c>
+      <c r="P28" s="4" t="s">
+        <v>641</v>
+      </c>
       <c r="Q28" s="4" t="s">
         <v>57</v>
       </c>
@@ -5394,9 +5517,11 @@
         <v>489</v>
       </c>
       <c r="O29" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P29" s="4"/>
+        <v>641</v>
+      </c>
+      <c r="P29" s="4" t="s">
+        <v>642</v>
+      </c>
       <c r="Q29" s="4" t="s">
         <v>57</v>
       </c>
@@ -5465,9 +5590,11 @@
         <v>491</v>
       </c>
       <c r="O30" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P30" s="4"/>
+        <v>643</v>
+      </c>
+      <c r="P30" s="4" t="s">
+        <v>644</v>
+      </c>
       <c r="Q30" s="4" t="s">
         <v>57</v>
       </c>
@@ -5534,7 +5661,7 @@
         <v>493</v>
       </c>
       <c r="O31" s="4" t="s">
-        <v>57</v>
+        <v>645</v>
       </c>
       <c r="P31" s="4"/>
       <c r="Q31" s="4" t="s">
@@ -5603,9 +5730,11 @@
         <v>495</v>
       </c>
       <c r="O32" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P32" s="4"/>
+        <v>645</v>
+      </c>
+      <c r="P32" s="4" t="s">
+        <v>646</v>
+      </c>
       <c r="Q32" s="4" t="s">
         <v>57</v>
       </c>
@@ -5672,9 +5801,11 @@
         <v>497</v>
       </c>
       <c r="O33" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P33" s="4"/>
+        <v>645</v>
+      </c>
+      <c r="P33" s="4" t="s">
+        <v>637</v>
+      </c>
       <c r="Q33" s="4" t="s">
         <v>57</v>
       </c>
@@ -5743,9 +5874,11 @@
         <v>499</v>
       </c>
       <c r="O34" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P34" s="4"/>
+        <v>647</v>
+      </c>
+      <c r="P34" s="4" t="s">
+        <v>641</v>
+      </c>
       <c r="Q34" s="4" t="s">
         <v>57</v>
       </c>
@@ -5812,7 +5945,7 @@
         <v>501</v>
       </c>
       <c r="O35" s="4" t="s">
-        <v>57</v>
+        <v>647</v>
       </c>
       <c r="P35" s="4"/>
       <c r="Q35" s="4" t="s">
@@ -5883,7 +6016,7 @@
         <v>503</v>
       </c>
       <c r="O36" s="4" t="s">
-        <v>57</v>
+        <v>641</v>
       </c>
       <c r="P36" s="4"/>
       <c r="Q36" s="4" t="s">
@@ -5954,9 +6087,11 @@
         <v>504</v>
       </c>
       <c r="O37" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P37" s="4"/>
+        <v>641</v>
+      </c>
+      <c r="P37" s="4" t="s">
+        <v>647</v>
+      </c>
       <c r="Q37" s="4" t="s">
         <v>57</v>
       </c>
@@ -6025,9 +6160,11 @@
         <v>506</v>
       </c>
       <c r="O38" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P38" s="4"/>
+        <v>629</v>
+      </c>
+      <c r="P38" s="4" t="s">
+        <v>625</v>
+      </c>
       <c r="Q38" s="4" t="s">
         <v>57</v>
       </c>
@@ -6094,7 +6231,7 @@
         <v>508</v>
       </c>
       <c r="O39" s="4" t="s">
-        <v>57</v>
+        <v>628</v>
       </c>
       <c r="P39" s="4"/>
       <c r="Q39" s="4" t="s">
@@ -6165,9 +6302,11 @@
         <v>510</v>
       </c>
       <c r="O40" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P40" s="4"/>
+        <v>648</v>
+      </c>
+      <c r="P40" s="4" t="s">
+        <v>649</v>
+      </c>
       <c r="Q40" s="4" t="s">
         <v>57</v>
       </c>
@@ -6236,9 +6375,11 @@
         <v>512</v>
       </c>
       <c r="O41" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P41" s="4"/>
+        <v>648</v>
+      </c>
+      <c r="P41" s="4" t="s">
+        <v>621</v>
+      </c>
       <c r="Q41" s="4" t="s">
         <v>57</v>
       </c>
@@ -6307,9 +6448,11 @@
         <v>514</v>
       </c>
       <c r="O42" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P42" s="4"/>
+        <v>629</v>
+      </c>
+      <c r="P42" s="4" t="s">
+        <v>650</v>
+      </c>
       <c r="Q42" s="4" t="s">
         <v>57</v>
       </c>
@@ -6376,9 +6519,11 @@
         <v>516</v>
       </c>
       <c r="O43" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P43" s="4"/>
+        <v>620</v>
+      </c>
+      <c r="P43" s="4" t="s">
+        <v>651</v>
+      </c>
       <c r="Q43" s="4" t="s">
         <v>57</v>
       </c>
@@ -6445,9 +6590,11 @@
         <v>518</v>
       </c>
       <c r="O44" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P44" s="4"/>
+        <v>620</v>
+      </c>
+      <c r="P44" s="4" t="s">
+        <v>629</v>
+      </c>
       <c r="Q44" s="4" t="s">
         <v>57</v>
       </c>
@@ -6516,9 +6663,11 @@
         <v>520</v>
       </c>
       <c r="O45" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P45" s="4"/>
+        <v>629</v>
+      </c>
+      <c r="P45" s="4" t="s">
+        <v>653</v>
+      </c>
       <c r="Q45" s="4" t="s">
         <v>57</v>
       </c>
@@ -6585,9 +6734,11 @@
         <v>522</v>
       </c>
       <c r="O46" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P46" s="4"/>
+        <v>652</v>
+      </c>
+      <c r="P46" s="4" t="s">
+        <v>654</v>
+      </c>
       <c r="Q46" s="4" t="s">
         <v>57</v>
       </c>
@@ -6654,9 +6805,11 @@
         <v>524</v>
       </c>
       <c r="O47" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P47" s="4"/>
+        <v>648</v>
+      </c>
+      <c r="P47" s="4" t="s">
+        <v>655</v>
+      </c>
       <c r="Q47" s="4" t="s">
         <v>57</v>
       </c>
@@ -6723,9 +6876,11 @@
         <v>526</v>
       </c>
       <c r="O48" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P48" s="4"/>
+        <v>628</v>
+      </c>
+      <c r="P48" s="4" t="s">
+        <v>621</v>
+      </c>
       <c r="Q48" s="4" t="s">
         <v>57</v>
       </c>
@@ -6794,9 +6949,11 @@
         <v>528</v>
       </c>
       <c r="O49" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P49" s="4"/>
+        <v>648</v>
+      </c>
+      <c r="P49" s="4" t="s">
+        <v>656</v>
+      </c>
       <c r="Q49" s="4" t="s">
         <v>57</v>
       </c>
@@ -6865,9 +7022,11 @@
         <v>530</v>
       </c>
       <c r="O50" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P50" s="4"/>
+        <v>641</v>
+      </c>
+      <c r="P50" s="4" t="s">
+        <v>657</v>
+      </c>
       <c r="Q50" s="4" t="s">
         <v>57</v>
       </c>
@@ -6934,9 +7093,11 @@
         <v>532</v>
       </c>
       <c r="O51" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P51" s="4"/>
+        <v>620</v>
+      </c>
+      <c r="P51" s="4" t="s">
+        <v>631</v>
+      </c>
       <c r="Q51" s="4" t="s">
         <v>57</v>
       </c>
@@ -7003,9 +7164,11 @@
         <v>534</v>
       </c>
       <c r="O52" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P52" s="4"/>
+        <v>641</v>
+      </c>
+      <c r="P52" s="4" t="s">
+        <v>658</v>
+      </c>
       <c r="Q52" s="4" t="s">
         <v>57</v>
       </c>
@@ -7074,9 +7237,11 @@
         <v>536</v>
       </c>
       <c r="O53" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P53" s="4"/>
+        <v>641</v>
+      </c>
+      <c r="P53" s="4" t="s">
+        <v>652</v>
+      </c>
       <c r="Q53" s="4" t="s">
         <v>57</v>
       </c>
@@ -7145,9 +7310,11 @@
         <v>538</v>
       </c>
       <c r="O54" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P54" s="4"/>
+        <v>622</v>
+      </c>
+      <c r="P54" s="4" t="s">
+        <v>659</v>
+      </c>
       <c r="Q54" s="4" t="s">
         <v>57</v>
       </c>
@@ -7214,9 +7381,11 @@
         <v>540</v>
       </c>
       <c r="O55" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P55" s="4"/>
+        <v>648</v>
+      </c>
+      <c r="P55" s="4" t="s">
+        <v>660</v>
+      </c>
       <c r="Q55" s="4" t="s">
         <v>57</v>
       </c>
@@ -7285,9 +7454,11 @@
         <v>542</v>
       </c>
       <c r="O56" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P56" s="4"/>
+        <v>629</v>
+      </c>
+      <c r="P56" s="4" t="s">
+        <v>628</v>
+      </c>
       <c r="Q56" s="4" t="s">
         <v>57</v>
       </c>
@@ -7354,9 +7525,11 @@
         <v>544</v>
       </c>
       <c r="O57" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P57" s="4"/>
+        <v>652</v>
+      </c>
+      <c r="P57" s="4" t="s">
+        <v>654</v>
+      </c>
       <c r="Q57" s="4" t="s">
         <v>57</v>
       </c>
@@ -7425,9 +7598,11 @@
         <v>546</v>
       </c>
       <c r="O58" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P58" s="4"/>
+        <v>641</v>
+      </c>
+      <c r="P58" s="4" t="s">
+        <v>661</v>
+      </c>
       <c r="Q58" s="4" t="s">
         <v>57</v>
       </c>
@@ -7496,9 +7671,11 @@
         <v>548</v>
       </c>
       <c r="O59" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P59" s="4"/>
+        <v>620</v>
+      </c>
+      <c r="P59" s="4" t="s">
+        <v>662</v>
+      </c>
       <c r="Q59" s="4" t="s">
         <v>57</v>
       </c>
@@ -7565,7 +7742,7 @@
         <v>508</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>57</v>
+        <v>628</v>
       </c>
       <c r="P60" s="6"/>
       <c r="Q60" s="6" t="s">
@@ -7597,13 +7774,28 @@
     <mergeCell ref="B1:Y1"/>
     <mergeCell ref="B2:Y2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:Y60">
-    <cfRule type="expression" dxfId="2" priority="1">
+  <conditionalFormatting sqref="A5:Y27 A29:O29 Q28:Y29 A28:N28 A30:Y33 A34:O34 Q34:Y34 A35:Y60">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>$E5="Must"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W5:W60">
-    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="Pending"/>
+    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="Pending"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P29">
+    <cfRule type="expression" dxfId="2" priority="8">
+      <formula>$E28="Must"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O28:P28">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$E28="Must"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P34">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$E34="Must"</formula>
+    </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" sqref="B5:B60" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -7629,20 +7821,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="27.95" customHeight="1">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="46" t="s">
         <v>284</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
     </row>
     <row r="2" spans="1:4" ht="21" customHeight="1">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="47" t="s">
         <v>285</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
     </row>
     <row r="4" spans="1:4" ht="15">
       <c r="A4" s="11" t="s">
@@ -7855,12 +8047,12 @@
       </c>
     </row>
     <row r="20" spans="1:4" ht="42" customHeight="1">
-      <c r="A20" s="45" t="s">
+      <c r="A20" s="48" t="s">
         <v>330</v>
       </c>
-      <c r="B20" s="46"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="47"/>
+      <c r="B20" s="49"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -8077,22 +8269,22 @@
   <sheetFormatPr defaultColWidth="66.875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.625" style="48" customWidth="1"/>
-    <col min="3" max="3" width="84.25" style="48" customWidth="1"/>
+    <col min="2" max="2" width="33.625" style="43" customWidth="1"/>
+    <col min="3" max="3" width="84.25" style="43" customWidth="1"/>
     <col min="4" max="4" width="33.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="44" t="s">
         <v>550</v>
       </c>
-      <c r="B1" s="50" t="s">
+      <c r="B1" s="45" t="s">
         <v>296</v>
       </c>
-      <c r="C1" s="50" t="s">
+      <c r="C1" s="45" t="s">
         <v>551</v>
       </c>
-      <c r="D1" s="49" t="s">
+      <c r="D1" s="44" t="s">
         <v>389</v>
       </c>
     </row>
@@ -8100,10 +8292,10 @@
       <c r="A2" t="s">
         <v>552</v>
       </c>
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="43" t="s">
         <v>553</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="43" t="s">
         <v>554</v>
       </c>
       <c r="D2" t="s">
@@ -8114,24 +8306,24 @@
       <c r="A3" t="s">
         <v>555</v>
       </c>
-      <c r="B3" s="48" t="s">
+      <c r="B3" s="43" t="s">
         <v>556</v>
       </c>
-      <c r="C3" s="48" t="s">
+      <c r="C3" s="43" t="s">
         <v>557</v>
       </c>
       <c r="D3" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" ht="28.5">
       <c r="A4" t="s">
         <v>558</v>
       </c>
-      <c r="B4" s="48" t="s">
+      <c r="B4" s="43" t="s">
         <v>559</v>
       </c>
-      <c r="C4" s="48" t="s">
+      <c r="C4" s="43" t="s">
         <v>560</v>
       </c>
       <c r="D4" t="s">
@@ -8142,10 +8334,10 @@
       <c r="A5" t="s">
         <v>561</v>
       </c>
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="43" t="s">
         <v>562</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="C5" s="43" t="s">
         <v>563</v>
       </c>
       <c r="D5" t="s">
@@ -8156,10 +8348,10 @@
       <c r="A6" t="s">
         <v>564</v>
       </c>
-      <c r="B6" s="48" t="s">
+      <c r="B6" s="43" t="s">
         <v>565</v>
       </c>
-      <c r="C6" s="48" t="s">
+      <c r="C6" s="43" t="s">
         <v>566</v>
       </c>
       <c r="D6" t="s">
@@ -8170,24 +8362,24 @@
       <c r="A7" t="s">
         <v>567</v>
       </c>
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="43" t="s">
         <v>568</v>
       </c>
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="43" t="s">
         <v>569</v>
       </c>
       <c r="D7" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" ht="28.5">
       <c r="A8" t="s">
         <v>570</v>
       </c>
-      <c r="B8" s="48" t="s">
+      <c r="B8" s="43" t="s">
         <v>571</v>
       </c>
-      <c r="C8" s="48" t="s">
+      <c r="C8" s="43" t="s">
         <v>572</v>
       </c>
       <c r="D8" t="s">
@@ -8198,10 +8390,10 @@
       <c r="A9" t="s">
         <v>573</v>
       </c>
-      <c r="B9" s="48" t="s">
+      <c r="B9" s="43" t="s">
         <v>574</v>
       </c>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="43" t="s">
         <v>575</v>
       </c>
       <c r="D9" t="s">
@@ -8212,10 +8404,10 @@
       <c r="A10" t="s">
         <v>576</v>
       </c>
-      <c r="B10" s="48" t="s">
+      <c r="B10" s="43" t="s">
         <v>577</v>
       </c>
-      <c r="C10" s="48" t="s">
+      <c r="C10" s="43" t="s">
         <v>578</v>
       </c>
       <c r="D10" t="s">
@@ -8226,10 +8418,10 @@
       <c r="A11" t="s">
         <v>579</v>
       </c>
-      <c r="B11" s="48" t="s">
+      <c r="B11" s="43" t="s">
         <v>580</v>
       </c>
-      <c r="C11" s="48" t="s">
+      <c r="C11" s="43" t="s">
         <v>581</v>
       </c>
       <c r="D11" t="s">
@@ -8240,10 +8432,10 @@
       <c r="A12" t="s">
         <v>582</v>
       </c>
-      <c r="B12" s="48" t="s">
+      <c r="B12" s="43" t="s">
         <v>583</v>
       </c>
-      <c r="C12" s="48" t="s">
+      <c r="C12" s="43" t="s">
         <v>584</v>
       </c>
       <c r="D12" t="s">
@@ -8254,24 +8446,24 @@
       <c r="A13" t="s">
         <v>585</v>
       </c>
-      <c r="B13" s="48" t="s">
+      <c r="B13" s="43" t="s">
         <v>586</v>
       </c>
-      <c r="C13" s="48" t="s">
+      <c r="C13" s="43" t="s">
         <v>587</v>
       </c>
       <c r="D13" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" ht="28.5">
       <c r="A14" t="s">
         <v>588</v>
       </c>
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="43" t="s">
         <v>589</v>
       </c>
-      <c r="C14" s="48" t="s">
+      <c r="C14" s="43" t="s">
         <v>590</v>
       </c>
       <c r="D14" t="s">
@@ -8282,10 +8474,10 @@
       <c r="A15" t="s">
         <v>591</v>
       </c>
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="43" t="s">
         <v>592</v>
       </c>
-      <c r="C15" s="48" t="s">
+      <c r="C15" s="43" t="s">
         <v>593</v>
       </c>
       <c r="D15" t="s">
@@ -8296,10 +8488,10 @@
       <c r="A16" t="s">
         <v>594</v>
       </c>
-      <c r="B16" s="48" t="s">
+      <c r="B16" s="43" t="s">
         <v>595</v>
       </c>
-      <c r="C16" s="48" t="s">
+      <c r="C16" s="43" t="s">
         <v>596</v>
       </c>
       <c r="D16" t="s">
@@ -8310,10 +8502,10 @@
       <c r="A17" t="s">
         <v>597</v>
       </c>
-      <c r="B17" s="48" t="s">
+      <c r="B17" s="43" t="s">
         <v>598</v>
       </c>
-      <c r="C17" s="48" t="s">
+      <c r="C17" s="43" t="s">
         <v>599</v>
       </c>
       <c r="D17" t="s">
@@ -8324,10 +8516,10 @@
       <c r="A18" t="s">
         <v>600</v>
       </c>
-      <c r="B18" s="48" t="s">
+      <c r="B18" s="43" t="s">
         <v>601</v>
       </c>
-      <c r="C18" s="48" t="s">
+      <c r="C18" s="43" t="s">
         <v>602</v>
       </c>
       <c r="D18" t="s">
@@ -8338,10 +8530,10 @@
       <c r="A19" t="s">
         <v>603</v>
       </c>
-      <c r="B19" s="48" t="s">
+      <c r="B19" s="43" t="s">
         <v>604</v>
       </c>
-      <c r="C19" s="48" t="s">
+      <c r="C19" s="43" t="s">
         <v>605</v>
       </c>
       <c r="D19" t="s">
@@ -8352,10 +8544,10 @@
       <c r="A20" t="s">
         <v>606</v>
       </c>
-      <c r="B20" s="48" t="s">
+      <c r="B20" s="43" t="s">
         <v>607</v>
       </c>
-      <c r="C20" s="48" t="s">
+      <c r="C20" s="43" t="s">
         <v>608</v>
       </c>
       <c r="D20" t="s">

</xml_diff>

<commit_message>
Low level design work. Documented LL design decision process regarding network segmentation, vm mapping and estate, dependencies. Delivered final LLDv1 doc outlining the LLD decisions which can be used to derive the Sprint backlog and Sprint planning.
</commit_message>
<xml_diff>
--- a/docs/project-management/02_Business_Requirements/Northwind-Outdoor-RTM-v1.0.xlsx
+++ b/docs/project-management/02_Business_Requirements/Northwind-Outdoor-RTM-v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/docs/project-management/02_Business_Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="740" documentId="8_{170D4D7C-E242-4887-90C6-7A678B36976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D54EF7AD-19F9-4EF6-9BB7-D46AC06A5B15}"/>
+  <xr:revisionPtr revIDLastSave="784" documentId="8_{170D4D7C-E242-4887-90C6-7A678B36976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30CC72D7-AC51-4E30-8460-6C0F686F2BF5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1509" uniqueCount="663">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1511" uniqueCount="667">
   <si>
     <t>Northwind Outdoor Ltd. | RTM Summary</t>
   </si>
@@ -2060,6 +2060,18 @@
   </si>
   <si>
     <t>DD-005 — Backup &amp; Recovery Architecture; DD-010 — Patch &amp; Software Lifecycle Management Architecture</t>
+  </si>
+  <si>
+    <t>LLD-01</t>
+  </si>
+  <si>
+    <t>LLD (Primary)</t>
+  </si>
+  <si>
+    <t>LLD (Secondary)</t>
+  </si>
+  <si>
+    <t>LLD-08</t>
   </si>
 </sst>
 </file>
@@ -2643,7 +2655,24 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="13">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2667,20 +2696,37 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color auto="1"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFDCE6F1"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFDCE6F1"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFDCE6F1"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFDCE6F1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -3142,8 +3188,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="RTMTable" displayName="RTMTable" ref="B4:Y60" totalsRowShown="0">
-  <tableColumns count="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="RTMTable" displayName="RTMTable" ref="B4:Z60" totalsRowShown="0">
+  <autoFilter ref="B4:Z60" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
+  <tableColumns count="25">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Requirement ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Type"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Requirement / Title"/>
@@ -3152,17 +3199,18 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="DF"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="BD"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="CAP (Primary)"/>
-    <tableColumn id="23" xr3:uid="{C116EC89-8261-41A9-893A-12DFD9AC01D5}" name="CAP (Secondary)" dataDxfId="11"/>
+    <tableColumn id="23" xr3:uid="{C116EC89-8261-41A9-893A-12DFD9AC01D5}" name="CAP (Secondary)" dataDxfId="12"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="BRD"/>
-    <tableColumn id="20" xr3:uid="{D1E0B300-86BD-45A9-B3EB-8951F17E8029}" name="Primary AD" dataDxfId="10"/>
-    <tableColumn id="22" xr3:uid="{701B3B8E-55FF-4520-83AD-295760593E66}" name="Key ADs" dataDxfId="9"/>
-    <tableColumn id="21" xr3:uid="{1638868F-A11C-40F1-8FB2-2AB197E42B79}" name="Secondary Ads" dataDxfId="8"/>
+    <tableColumn id="20" xr3:uid="{D1E0B300-86BD-45A9-B3EB-8951F17E8029}" name="Primary AD" dataDxfId="11"/>
+    <tableColumn id="22" xr3:uid="{701B3B8E-55FF-4520-83AD-295760593E66}" name="Key ADs" dataDxfId="10"/>
+    <tableColumn id="21" xr3:uid="{1638868F-A11C-40F1-8FB2-2AB197E42B79}" name="Secondary Ads" dataDxfId="9"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="HLD (Primary)"/>
-    <tableColumn id="24" xr3:uid="{599BD185-8391-4930-BB9A-B52E39596ACD}" name="HLD (Secondary)" dataDxfId="7"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="LLD"/>
+    <tableColumn id="24" xr3:uid="{599BD185-8391-4930-BB9A-B52E39596ACD}" name="HLD (Secondary)" dataDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="LLD (Primary)"/>
+    <tableColumn id="10" xr3:uid="{D9149C79-EC24-41C1-B36D-CD2D9225FFA3}" name="LLD (Secondary)" dataDxfId="5"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="ADR"/>
-    <tableColumn id="25" xr3:uid="{28378BB4-B208-482C-96C2-5A1994DECC42}" name="SOW" dataDxfId="6"/>
-    <tableColumn id="26" xr3:uid="{BAEC8EC4-D90B-4FBA-979D-21CDBE3C330A}" name="Sprint" dataDxfId="5"/>
+    <tableColumn id="25" xr3:uid="{28378BB4-B208-482C-96C2-5A1994DECC42}" name="SOW" dataDxfId="7"/>
+    <tableColumn id="26" xr3:uid="{BAEC8EC4-D90B-4FBA-979D-21CDBE3C330A}" name="Sprint" dataDxfId="6"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Test / UAT"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Acceptance Criteria"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Status"/>
@@ -3578,7 +3626,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="32">
-        <f>COUNTIF(RTM!$W$5:$W$60,A16)</f>
+        <f>COUNTIF(RTM!$X$5:$X$60,A16)</f>
         <v>56</v>
       </c>
     </row>
@@ -3594,7 +3642,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Y60"/>
+  <dimension ref="A1:Z60"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14.625" bestFit="1" customWidth="1"/>
@@ -3613,16 +3661,18 @@
     <col min="14" max="14" width="15.625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="11.5" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="26.375" customWidth="1"/>
-    <col min="17" max="18" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="11.5" customWidth="1"/>
-    <col min="21" max="21" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="42" customWidth="1"/>
-    <col min="23" max="23" width="19.625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="25" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="54" customWidth="1"/>
+    <col min="17" max="17" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.5" customWidth="1"/>
+    <col min="19" max="19" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="11.5" customWidth="1"/>
+    <col min="22" max="22" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="42" customWidth="1"/>
+    <col min="24" max="24" width="19.625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="25" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="54" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="27.95" customHeight="1">
+    <row r="1" spans="1:26" ht="27.95" customHeight="1">
       <c r="B1" s="46" t="s">
         <v>32</v>
       </c>
@@ -3649,8 +3699,9 @@
       <c r="W1" s="46"/>
       <c r="X1" s="46"/>
       <c r="Y1" s="46"/>
-    </row>
-    <row r="2" spans="1:25" ht="21" customHeight="1">
+      <c r="Z1" s="46"/>
+    </row>
+    <row r="2" spans="1:26" ht="21" customHeight="1">
       <c r="B2" s="47" t="s">
         <v>33</v>
       </c>
@@ -3677,8 +3728,9 @@
       <c r="W2" s="47"/>
       <c r="X2" s="47"/>
       <c r="Y2" s="47"/>
-    </row>
-    <row r="4" spans="1:25" ht="33" customHeight="1">
+      <c r="Z2" s="47"/>
+    </row>
+    <row r="4" spans="1:26" ht="33" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>387</v>
       </c>
@@ -3728,34 +3780,37 @@
         <v>624</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>46</v>
+        <v>664</v>
       </c>
       <c r="R4" s="1" t="s">
+        <v>665</v>
+      </c>
+      <c r="S4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="S4" s="1" t="s">
+      <c r="T4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="T4" s="1" t="s">
+      <c r="U4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="U4" s="1" t="s">
+      <c r="V4" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="V4" s="1" t="s">
+      <c r="W4" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="W4" s="1" t="s">
+      <c r="X4" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="X4" s="1" t="s">
+      <c r="Y4" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="Y4" s="1" t="s">
+      <c r="Z4" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="51.95" customHeight="1">
+    <row r="5" spans="1:26" ht="51.95" customHeight="1">
       <c r="A5" s="39" t="s">
         <v>57</v>
       </c>
@@ -3803,28 +3858,29 @@
       <c r="Q5" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="R5" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="S5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="T5" s="2"/>
-      <c r="U5" s="2" t="s">
-        <v>57</v>
-      </c>
+      <c r="U5" s="2"/>
       <c r="V5" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="W5" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="W5" s="2" t="s">
+      <c r="X5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="X5" s="2" t="s">
+      <c r="Y5" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="Y5" s="3" t="s">
+      <c r="Z5" s="3" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="51.95" customHeight="1">
+    <row r="6" spans="1:26" ht="51.95" customHeight="1">
       <c r="A6" s="39" t="s">
         <v>57</v>
       </c>
@@ -3872,28 +3928,29 @@
       <c r="Q6" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R6" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T6" s="4"/>
-      <c r="U6" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U6" s="4"/>
       <c r="V6" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W6" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="W6" s="4" t="s">
+      <c r="X6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X6" s="4" t="s">
+      <c r="Y6" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y6" s="5" t="s">
+      <c r="Z6" s="5" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="51.95" customHeight="1">
+    <row r="7" spans="1:26" ht="51.95" customHeight="1">
       <c r="A7" s="39" t="s">
         <v>57</v>
       </c>
@@ -3941,28 +3998,29 @@
       <c r="Q7" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R7" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S7" s="4"/>
+      <c r="R7" s="4"/>
+      <c r="S7" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T7" s="4"/>
-      <c r="U7" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U7" s="4"/>
       <c r="V7" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W7" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="W7" s="4" t="s">
+      <c r="X7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X7" s="4" t="s">
+      <c r="Y7" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y7" s="5" t="s">
+      <c r="Z7" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="51.95" customHeight="1">
+    <row r="8" spans="1:26" ht="51.95" customHeight="1">
       <c r="A8" s="39" t="s">
         <v>57</v>
       </c>
@@ -4012,28 +4070,29 @@
       <c r="Q8" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R8" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T8" s="4"/>
-      <c r="U8" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U8" s="4"/>
       <c r="V8" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W8" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="W8" s="4" t="s">
+      <c r="X8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X8" s="4" t="s">
+      <c r="Y8" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y8" s="5" t="s">
+      <c r="Z8" s="5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="51.95" customHeight="1">
+    <row r="9" spans="1:26" ht="51.95" customHeight="1">
       <c r="A9" s="39" t="s">
         <v>57</v>
       </c>
@@ -4081,28 +4140,29 @@
       <c r="Q9" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R9" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S9" s="4"/>
+      <c r="R9" s="4"/>
+      <c r="S9" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T9" s="4"/>
-      <c r="U9" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U9" s="4"/>
       <c r="V9" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W9" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="W9" s="4" t="s">
+      <c r="X9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X9" s="4" t="s">
+      <c r="Y9" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y9" s="5" t="s">
+      <c r="Z9" s="5" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="51.95" customHeight="1">
+    <row r="10" spans="1:26" ht="51.95" customHeight="1">
       <c r="A10" s="39" t="s">
         <v>57</v>
       </c>
@@ -4154,28 +4214,29 @@
       <c r="Q10" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R10" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S10" s="4"/>
+      <c r="R10" s="4"/>
+      <c r="S10" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T10" s="4"/>
-      <c r="U10" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U10" s="4"/>
       <c r="V10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W10" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="W10" s="4" t="s">
+      <c r="X10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X10" s="4" t="s">
+      <c r="Y10" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y10" s="5" t="s">
+      <c r="Z10" s="5" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="51.95" customHeight="1">
+    <row r="11" spans="1:26" ht="51.95" customHeight="1">
       <c r="A11" s="39" t="s">
         <v>57</v>
       </c>
@@ -4225,28 +4286,29 @@
       <c r="Q11" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R11" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S11" s="4"/>
+      <c r="R11" s="4"/>
+      <c r="S11" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T11" s="4"/>
-      <c r="U11" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U11" s="4"/>
       <c r="V11" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W11" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="W11" s="4" t="s">
+      <c r="X11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X11" s="4" t="s">
+      <c r="Y11" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y11" s="5" t="s">
+      <c r="Z11" s="5" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="51.95" customHeight="1">
+    <row r="12" spans="1:26" ht="51.95" customHeight="1">
       <c r="A12" s="39" t="s">
         <v>57</v>
       </c>
@@ -4298,28 +4360,29 @@
       <c r="Q12" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R12" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S12" s="4"/>
+      <c r="R12" s="4"/>
+      <c r="S12" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T12" s="4"/>
-      <c r="U12" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U12" s="4"/>
       <c r="V12" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W12" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="W12" s="4" t="s">
+      <c r="X12" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X12" s="4" t="s">
+      <c r="Y12" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y12" s="5" t="s">
+      <c r="Z12" s="5" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="51.95" customHeight="1">
+    <row r="13" spans="1:26" ht="51.95" customHeight="1">
       <c r="A13" s="39" t="s">
         <v>57</v>
       </c>
@@ -4371,28 +4434,29 @@
       <c r="Q13" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R13" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S13" s="4"/>
+      <c r="R13" s="4"/>
+      <c r="S13" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T13" s="4"/>
-      <c r="U13" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U13" s="4"/>
       <c r="V13" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W13" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="W13" s="4" t="s">
+      <c r="X13" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X13" s="4" t="s">
+      <c r="Y13" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y13" s="5" t="s">
+      <c r="Z13" s="5" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="51.95" customHeight="1">
+    <row r="14" spans="1:26" ht="51.95" customHeight="1">
       <c r="A14" s="39" t="s">
         <v>57</v>
       </c>
@@ -4438,30 +4502,33 @@
       </c>
       <c r="P14" s="4"/>
       <c r="Q14" s="4" t="s">
-        <v>57</v>
+        <v>666</v>
       </c>
       <c r="R14" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S14" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="S14" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T14" s="4"/>
-      <c r="U14" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U14" s="4"/>
       <c r="V14" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W14" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="W14" s="4" t="s">
+      <c r="X14" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X14" s="4" t="s">
+      <c r="Y14" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y14" s="5" t="s">
+      <c r="Z14" s="5" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="51.95" customHeight="1">
+    <row r="15" spans="1:26" ht="51.95" customHeight="1">
       <c r="A15" s="39" t="s">
         <v>57</v>
       </c>
@@ -4510,31 +4577,32 @@
       <c r="P15" s="4" t="s">
         <v>628</v>
       </c>
-      <c r="Q15" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="Q15" s="4"/>
       <c r="R15" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S15" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="S15" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T15" s="4"/>
-      <c r="U15" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U15" s="4"/>
       <c r="V15" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W15" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="W15" s="4" t="s">
+      <c r="X15" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X15" s="4" t="s">
+      <c r="Y15" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y15" s="5" t="s">
+      <c r="Z15" s="5" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="51.95" customHeight="1">
+    <row r="16" spans="1:26" ht="51.95" customHeight="1">
       <c r="A16" s="39" t="s">
         <v>57</v>
       </c>
@@ -4586,28 +4654,29 @@
       <c r="Q16" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R16" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S16" s="4"/>
+      <c r="R16" s="4"/>
+      <c r="S16" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T16" s="4"/>
-      <c r="U16" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U16" s="4"/>
       <c r="V16" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W16" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="W16" s="4" t="s">
+      <c r="X16" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X16" s="4" t="s">
+      <c r="Y16" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y16" s="5" t="s">
+      <c r="Z16" s="5" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="17" spans="1:25" ht="51.95" customHeight="1">
+    <row r="17" spans="1:26" ht="51.95" customHeight="1">
       <c r="A17" s="39" t="s">
         <v>57</v>
       </c>
@@ -4656,31 +4725,32 @@
       <c r="P17" s="4" t="s">
         <v>620</v>
       </c>
-      <c r="Q17" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="Q17" s="4"/>
       <c r="R17" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S17" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="S17" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T17" s="4"/>
-      <c r="U17" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U17" s="4"/>
       <c r="V17" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W17" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="W17" s="4" t="s">
+      <c r="X17" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X17" s="4" t="s">
+      <c r="Y17" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y17" s="5" t="s">
+      <c r="Z17" s="5" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="18" spans="1:25" ht="51.95" customHeight="1">
+    <row r="18" spans="1:26" ht="51.95" customHeight="1">
       <c r="A18" s="39" t="s">
         <v>57</v>
       </c>
@@ -4729,31 +4799,32 @@
       <c r="P18" s="4" t="s">
         <v>620</v>
       </c>
-      <c r="Q18" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="Q18" s="4"/>
       <c r="R18" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S18" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="S18" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T18" s="4"/>
-      <c r="U18" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U18" s="4"/>
       <c r="V18" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W18" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="W18" s="4" t="s">
+      <c r="X18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X18" s="4" t="s">
+      <c r="Y18" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y18" s="5" t="s">
+      <c r="Z18" s="5" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="19" spans="1:25" ht="51.95" customHeight="1">
+    <row r="19" spans="1:26" ht="51.95" customHeight="1">
       <c r="A19" s="39" t="s">
         <v>57</v>
       </c>
@@ -4802,31 +4873,32 @@
       <c r="P19" s="4" t="s">
         <v>631</v>
       </c>
-      <c r="Q19" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="Q19" s="4"/>
       <c r="R19" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S19" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="S19" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T19" s="4"/>
-      <c r="U19" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U19" s="4"/>
       <c r="V19" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W19" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="W19" s="4" t="s">
+      <c r="X19" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X19" s="4" t="s">
+      <c r="Y19" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y19" s="5" t="s">
+      <c r="Z19" s="5" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="20" spans="1:25" ht="51.95" customHeight="1">
+    <row r="20" spans="1:26" ht="51.95" customHeight="1">
       <c r="A20" s="39" t="s">
         <v>57</v>
       </c>
@@ -4876,28 +4948,29 @@
       <c r="Q20" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R20" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S20" s="4"/>
+      <c r="R20" s="4"/>
+      <c r="S20" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T20" s="4"/>
-      <c r="U20" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U20" s="4"/>
       <c r="V20" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W20" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W20" s="4" t="s">
+      <c r="X20" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X20" s="4" t="s">
+      <c r="Y20" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y20" s="5" t="s">
+      <c r="Z20" s="5" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="21" spans="1:25" ht="51.95" customHeight="1">
+    <row r="21" spans="1:26" ht="51.95" customHeight="1">
       <c r="A21" s="39" t="s">
         <v>57</v>
       </c>
@@ -4947,30 +5020,31 @@
         <v>634</v>
       </c>
       <c r="Q21" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="R21" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S21" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="R21" s="4"/>
+      <c r="S21" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T21" s="4"/>
-      <c r="U21" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U21" s="4"/>
       <c r="V21" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W21" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="W21" s="4" t="s">
+      <c r="X21" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X21" s="4" t="s">
+      <c r="Y21" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y21" s="5" t="s">
+      <c r="Z21" s="5" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="22" spans="1:25" ht="51.95" customHeight="1">
+    <row r="22" spans="1:26" ht="51.95" customHeight="1">
       <c r="A22" s="39" t="s">
         <v>57</v>
       </c>
@@ -5022,28 +5096,29 @@
       <c r="Q22" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R22" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S22" s="4"/>
+      <c r="R22" s="4"/>
+      <c r="S22" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T22" s="4"/>
-      <c r="U22" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U22" s="4"/>
       <c r="V22" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W22" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="W22" s="4" t="s">
+      <c r="X22" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X22" s="4" t="s">
+      <c r="Y22" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y22" s="5" t="s">
+      <c r="Z22" s="5" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="23" spans="1:25" ht="51.95" customHeight="1">
+    <row r="23" spans="1:26" ht="51.95" customHeight="1">
       <c r="A23" s="39" t="s">
         <v>57</v>
       </c>
@@ -5093,30 +5168,31 @@
         <v>621</v>
       </c>
       <c r="Q23" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="R23" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S23" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="R23" s="4"/>
+      <c r="S23" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T23" s="4"/>
-      <c r="U23" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U23" s="4"/>
       <c r="V23" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W23" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="W23" s="4" t="s">
+      <c r="X23" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X23" s="4" t="s">
+      <c r="Y23" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y23" s="5" t="s">
+      <c r="Z23" s="5" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="24" spans="1:25" ht="51.95" customHeight="1">
+    <row r="24" spans="1:26" ht="51.95" customHeight="1">
       <c r="A24" s="39" t="s">
         <v>57</v>
       </c>
@@ -5166,30 +5242,31 @@
         <v>637</v>
       </c>
       <c r="Q24" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="R24" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S24" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="R24" s="4"/>
+      <c r="S24" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T24" s="4"/>
-      <c r="U24" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U24" s="4"/>
       <c r="V24" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W24" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="W24" s="4" t="s">
+      <c r="X24" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X24" s="4" t="s">
+      <c r="Y24" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y24" s="5" t="s">
+      <c r="Z24" s="5" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="25" spans="1:25" ht="51.95" customHeight="1">
+    <row r="25" spans="1:26" ht="51.95" customHeight="1">
       <c r="A25" s="39" t="s">
         <v>57</v>
       </c>
@@ -5237,28 +5314,29 @@
       <c r="Q25" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R25" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S25" s="4"/>
+      <c r="R25" s="4"/>
+      <c r="S25" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T25" s="4"/>
-      <c r="U25" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U25" s="4"/>
       <c r="V25" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W25" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="W25" s="4" t="s">
+      <c r="X25" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X25" s="4" t="s">
+      <c r="Y25" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y25" s="5" t="s">
+      <c r="Z25" s="5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="26" spans="1:25" ht="51.95" customHeight="1">
+    <row r="26" spans="1:26" ht="51.95" customHeight="1">
       <c r="A26" s="39" t="s">
         <v>57</v>
       </c>
@@ -5310,28 +5388,29 @@
       <c r="Q26" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R26" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S26" s="4"/>
+      <c r="R26" s="4"/>
+      <c r="S26" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T26" s="4"/>
-      <c r="U26" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U26" s="4"/>
       <c r="V26" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W26" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="W26" s="4" t="s">
+      <c r="X26" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X26" s="4" t="s">
+      <c r="Y26" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y26" s="5" t="s">
+      <c r="Z26" s="5" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="27" spans="1:25" ht="51.95" customHeight="1">
+    <row r="27" spans="1:26" ht="51.95" customHeight="1">
       <c r="A27" s="39" t="s">
         <v>57</v>
       </c>
@@ -5379,30 +5458,31 @@
         <v>640</v>
       </c>
       <c r="Q27" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="R27" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S27" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="R27" s="4"/>
+      <c r="S27" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T27" s="4"/>
-      <c r="U27" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U27" s="4"/>
       <c r="V27" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W27" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="W27" s="4" t="s">
+      <c r="X27" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X27" s="4" t="s">
+      <c r="Y27" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y27" s="5" t="s">
+      <c r="Z27" s="5" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="28" spans="1:25" ht="51.95" customHeight="1">
+    <row r="28" spans="1:26" ht="51.95" customHeight="1">
       <c r="A28" s="39" t="s">
         <v>57</v>
       </c>
@@ -5452,30 +5532,31 @@
         <v>641</v>
       </c>
       <c r="Q28" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="R28" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S28" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="R28" s="4"/>
+      <c r="S28" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T28" s="4"/>
-      <c r="U28" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U28" s="4"/>
       <c r="V28" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W28" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="W28" s="4" t="s">
+      <c r="X28" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X28" s="4" t="s">
+      <c r="Y28" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y28" s="5" t="s">
+      <c r="Z28" s="5" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="29" spans="1:25" ht="51.95" customHeight="1">
+    <row r="29" spans="1:26" ht="51.95" customHeight="1">
       <c r="A29" s="39" t="s">
         <v>57</v>
       </c>
@@ -5525,28 +5606,29 @@
       <c r="Q29" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R29" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S29" s="4"/>
+      <c r="R29" s="4"/>
+      <c r="S29" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T29" s="4"/>
-      <c r="U29" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U29" s="4"/>
       <c r="V29" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W29" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="W29" s="4" t="s">
+      <c r="X29" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X29" s="4" t="s">
+      <c r="Y29" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y29" s="5" t="s">
+      <c r="Z29" s="5" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="30" spans="1:25" ht="51.95" customHeight="1">
+    <row r="30" spans="1:26" ht="51.95" customHeight="1">
       <c r="A30" s="39" t="s">
         <v>57</v>
       </c>
@@ -5598,28 +5680,29 @@
       <c r="Q30" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R30" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S30" s="4"/>
+      <c r="R30" s="4"/>
+      <c r="S30" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T30" s="4"/>
-      <c r="U30" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U30" s="4"/>
       <c r="V30" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W30" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="W30" s="4" t="s">
+      <c r="X30" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X30" s="4" t="s">
+      <c r="Y30" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y30" s="5" t="s">
+      <c r="Z30" s="5" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="31" spans="1:25" ht="51.95" customHeight="1">
+    <row r="31" spans="1:26" ht="51.95" customHeight="1">
       <c r="A31" s="39" t="s">
         <v>57</v>
       </c>
@@ -5667,28 +5750,29 @@
       <c r="Q31" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R31" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S31" s="4"/>
+      <c r="R31" s="4"/>
+      <c r="S31" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T31" s="4"/>
-      <c r="U31" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U31" s="4"/>
       <c r="V31" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W31" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="W31" s="4" t="s">
+      <c r="X31" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X31" s="4" t="s">
+      <c r="Y31" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y31" s="5" t="s">
+      <c r="Z31" s="5" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="32" spans="1:25" ht="51.95" customHeight="1">
+    <row r="32" spans="1:26" ht="51.95" customHeight="1">
       <c r="A32" s="39" t="s">
         <v>57</v>
       </c>
@@ -5738,28 +5822,29 @@
       <c r="Q32" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R32" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S32" s="4"/>
+      <c r="R32" s="4"/>
+      <c r="S32" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T32" s="4"/>
-      <c r="U32" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U32" s="4"/>
       <c r="V32" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W32" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="W32" s="4" t="s">
+      <c r="X32" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X32" s="4" t="s">
+      <c r="Y32" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y32" s="5" t="s">
+      <c r="Z32" s="5" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="33" spans="1:25" ht="51.95" customHeight="1">
+    <row r="33" spans="1:26" ht="51.95" customHeight="1">
       <c r="A33" s="39" t="s">
         <v>57</v>
       </c>
@@ -5809,28 +5894,29 @@
       <c r="Q33" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R33" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S33" s="4"/>
+      <c r="R33" s="4"/>
+      <c r="S33" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T33" s="4"/>
-      <c r="U33" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U33" s="4"/>
       <c r="V33" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W33" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="W33" s="4" t="s">
+      <c r="X33" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X33" s="4" t="s">
+      <c r="Y33" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y33" s="5" t="s">
+      <c r="Z33" s="5" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:25" ht="51.95" customHeight="1">
+    <row r="34" spans="1:26" ht="51.95" customHeight="1">
       <c r="A34" s="39" t="s">
         <v>57</v>
       </c>
@@ -5882,28 +5968,29 @@
       <c r="Q34" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R34" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S34" s="4"/>
+      <c r="R34" s="4"/>
+      <c r="S34" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T34" s="4"/>
-      <c r="U34" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U34" s="4"/>
       <c r="V34" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W34" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="W34" s="4" t="s">
+      <c r="X34" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X34" s="4" t="s">
+      <c r="Y34" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y34" s="5" t="s">
+      <c r="Z34" s="5" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="35" spans="1:25" ht="51.95" customHeight="1">
+    <row r="35" spans="1:26" ht="51.95" customHeight="1">
       <c r="A35" s="39" t="s">
         <v>57</v>
       </c>
@@ -5951,28 +6038,29 @@
       <c r="Q35" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R35" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S35" s="4"/>
+      <c r="R35" s="4"/>
+      <c r="S35" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T35" s="4"/>
-      <c r="U35" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U35" s="4"/>
       <c r="V35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W35" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="W35" s="4" t="s">
+      <c r="X35" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X35" s="4" t="s">
+      <c r="Y35" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y35" s="5" t="s">
+      <c r="Z35" s="5" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="36" spans="1:25" ht="51.95" customHeight="1">
+    <row r="36" spans="1:26" ht="51.95" customHeight="1">
       <c r="A36" s="39" t="s">
         <v>57</v>
       </c>
@@ -6022,28 +6110,29 @@
       <c r="Q36" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R36" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S36" s="4"/>
+      <c r="R36" s="4"/>
+      <c r="S36" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T36" s="4"/>
-      <c r="U36" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U36" s="4"/>
       <c r="V36" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W36" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="W36" s="4" t="s">
+      <c r="X36" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X36" s="4" t="s">
+      <c r="Y36" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y36" s="5" t="s">
+      <c r="Z36" s="5" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="37" spans="1:25" ht="51.95" customHeight="1">
+    <row r="37" spans="1:26" ht="51.95" customHeight="1">
       <c r="A37" s="39" t="s">
         <v>57</v>
       </c>
@@ -6095,28 +6184,29 @@
       <c r="Q37" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R37" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S37" s="4"/>
+      <c r="R37" s="4"/>
+      <c r="S37" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T37" s="4"/>
-      <c r="U37" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U37" s="4"/>
       <c r="V37" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W37" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="W37" s="4" t="s">
+      <c r="X37" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X37" s="4" t="s">
+      <c r="Y37" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y37" s="5" t="s">
+      <c r="Z37" s="5" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="38" spans="1:25" ht="51.95" customHeight="1">
+    <row r="38" spans="1:26" ht="51.95" customHeight="1">
       <c r="A38" s="39" t="s">
         <v>57</v>
       </c>
@@ -6165,31 +6255,32 @@
       <c r="P38" s="4" t="s">
         <v>625</v>
       </c>
-      <c r="Q38" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="Q38" s="4"/>
       <c r="R38" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S38" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="S38" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T38" s="4"/>
-      <c r="U38" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U38" s="4"/>
       <c r="V38" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W38" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="W38" s="4" t="s">
+      <c r="X38" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X38" s="4" t="s">
+      <c r="Y38" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y38" s="5" t="s">
+      <c r="Z38" s="5" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="39" spans="1:25" ht="51.95" customHeight="1">
+    <row r="39" spans="1:26" ht="51.95" customHeight="1">
       <c r="A39" s="39" t="s">
         <v>57</v>
       </c>
@@ -6234,31 +6325,32 @@
         <v>628</v>
       </c>
       <c r="P39" s="4"/>
-      <c r="Q39" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="Q39" s="4"/>
       <c r="R39" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S39" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="S39" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T39" s="4"/>
-      <c r="U39" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U39" s="4"/>
       <c r="V39" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W39" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="W39" s="4" t="s">
+      <c r="X39" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X39" s="4" t="s">
+      <c r="Y39" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y39" s="5" t="s">
+      <c r="Z39" s="5" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="40" spans="1:25" ht="51.95" customHeight="1">
+    <row r="40" spans="1:26" ht="51.95" customHeight="1">
       <c r="A40" s="39" t="s">
         <v>57</v>
       </c>
@@ -6310,28 +6402,29 @@
       <c r="Q40" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R40" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S40" s="4"/>
+      <c r="R40" s="4"/>
+      <c r="S40" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T40" s="4"/>
-      <c r="U40" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U40" s="4"/>
       <c r="V40" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W40" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="W40" s="4" t="s">
+      <c r="X40" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X40" s="4" t="s">
+      <c r="Y40" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y40" s="5" t="s">
+      <c r="Z40" s="5" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="41" spans="1:25" ht="51.95" customHeight="1">
+    <row r="41" spans="1:26" ht="51.95" customHeight="1">
       <c r="A41" s="39" t="s">
         <v>57</v>
       </c>
@@ -6381,30 +6474,31 @@
         <v>621</v>
       </c>
       <c r="Q41" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="R41" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S41" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="R41" s="4"/>
+      <c r="S41" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T41" s="4"/>
-      <c r="U41" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U41" s="4"/>
       <c r="V41" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W41" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="W41" s="4" t="s">
+      <c r="X41" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X41" s="4" t="s">
+      <c r="Y41" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y41" s="5" t="s">
+      <c r="Z41" s="5" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="42" spans="1:25" ht="51.95" customHeight="1">
+    <row r="42" spans="1:26" ht="51.95" customHeight="1">
       <c r="A42" s="39" t="s">
         <v>57</v>
       </c>
@@ -6456,28 +6550,29 @@
       <c r="Q42" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R42" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S42" s="4"/>
+      <c r="R42" s="4"/>
+      <c r="S42" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T42" s="4"/>
-      <c r="U42" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U42" s="4"/>
       <c r="V42" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W42" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="W42" s="4" t="s">
+      <c r="X42" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X42" s="4" t="s">
+      <c r="Y42" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y42" s="5" t="s">
+      <c r="Z42" s="5" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="43" spans="1:25" ht="51.95" customHeight="1">
+    <row r="43" spans="1:26" ht="51.95" customHeight="1">
       <c r="A43" s="39" t="s">
         <v>57</v>
       </c>
@@ -6527,28 +6622,29 @@
       <c r="Q43" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R43" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S43" s="4"/>
+      <c r="R43" s="4"/>
+      <c r="S43" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T43" s="4"/>
-      <c r="U43" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U43" s="4"/>
       <c r="V43" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W43" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="W43" s="4" t="s">
+      <c r="X43" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X43" s="4" t="s">
+      <c r="Y43" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y43" s="5" t="s">
+      <c r="Z43" s="5" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="44" spans="1:25" ht="51.95" customHeight="1">
+    <row r="44" spans="1:26" ht="51.95" customHeight="1">
       <c r="A44" s="39" t="s">
         <v>57</v>
       </c>
@@ -6596,30 +6692,31 @@
         <v>629</v>
       </c>
       <c r="Q44" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="R44" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S44" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="R44" s="4"/>
+      <c r="S44" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T44" s="4"/>
-      <c r="U44" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U44" s="4"/>
       <c r="V44" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W44" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="W44" s="4" t="s">
+      <c r="X44" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X44" s="4" t="s">
+      <c r="Y44" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y44" s="5" t="s">
+      <c r="Z44" s="5" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="45" spans="1:25" ht="51.95" customHeight="1">
+    <row r="45" spans="1:26" ht="51.95" customHeight="1">
       <c r="A45" s="39" t="s">
         <v>57</v>
       </c>
@@ -6669,30 +6766,31 @@
         <v>653</v>
       </c>
       <c r="Q45" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="R45" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S45" s="4"/>
+        <v>663</v>
+      </c>
+      <c r="R45" s="4"/>
+      <c r="S45" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T45" s="4"/>
-      <c r="U45" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U45" s="4"/>
       <c r="V45" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W45" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="W45" s="4" t="s">
+      <c r="X45" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X45" s="4" t="s">
+      <c r="Y45" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y45" s="5" t="s">
+      <c r="Z45" s="5" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="46" spans="1:25" ht="51.95" customHeight="1">
+    <row r="46" spans="1:26" ht="51.95" customHeight="1">
       <c r="A46" s="39" t="s">
         <v>57</v>
       </c>
@@ -6742,28 +6840,29 @@
       <c r="Q46" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R46" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S46" s="4"/>
+      <c r="R46" s="4"/>
+      <c r="S46" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T46" s="4"/>
-      <c r="U46" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U46" s="4"/>
       <c r="V46" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W46" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="W46" s="4" t="s">
+      <c r="X46" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X46" s="4" t="s">
+      <c r="Y46" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y46" s="5" t="s">
+      <c r="Z46" s="5" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="47" spans="1:25" ht="51.95" customHeight="1">
+    <row r="47" spans="1:26" ht="51.95" customHeight="1">
       <c r="A47" s="39" t="s">
         <v>57</v>
       </c>
@@ -6813,28 +6912,29 @@
       <c r="Q47" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R47" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S47" s="4"/>
+      <c r="R47" s="4"/>
+      <c r="S47" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T47" s="4"/>
-      <c r="U47" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U47" s="4"/>
       <c r="V47" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W47" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="W47" s="4" t="s">
+      <c r="X47" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X47" s="4" t="s">
+      <c r="Y47" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y47" s="5" t="s">
+      <c r="Z47" s="5" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="48" spans="1:25" ht="51.95" customHeight="1">
+    <row r="48" spans="1:26" ht="51.95" customHeight="1">
       <c r="A48" s="39" t="s">
         <v>57</v>
       </c>
@@ -6884,28 +6984,29 @@
       <c r="Q48" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R48" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S48" s="4"/>
+      <c r="R48" s="4"/>
+      <c r="S48" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T48" s="4"/>
-      <c r="U48" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U48" s="4"/>
       <c r="V48" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W48" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="W48" s="4" t="s">
+      <c r="X48" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X48" s="4" t="s">
+      <c r="Y48" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y48" s="5" t="s">
+      <c r="Z48" s="5" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="49" spans="1:25" ht="51.95" customHeight="1">
+    <row r="49" spans="1:26" ht="51.95" customHeight="1">
       <c r="A49" s="39" t="s">
         <v>57</v>
       </c>
@@ -6957,28 +7058,29 @@
       <c r="Q49" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R49" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S49" s="4"/>
+      <c r="R49" s="4"/>
+      <c r="S49" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T49" s="4"/>
-      <c r="U49" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U49" s="4"/>
       <c r="V49" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W49" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="W49" s="4" t="s">
+      <c r="X49" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X49" s="4" t="s">
+      <c r="Y49" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y49" s="5" t="s">
+      <c r="Z49" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="50" spans="1:25" ht="51.95" customHeight="1">
+    <row r="50" spans="1:26" ht="51.95" customHeight="1">
       <c r="A50" s="39" t="s">
         <v>57</v>
       </c>
@@ -7030,28 +7132,29 @@
       <c r="Q50" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R50" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S50" s="4"/>
+      <c r="R50" s="4"/>
+      <c r="S50" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T50" s="4"/>
-      <c r="U50" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U50" s="4"/>
       <c r="V50" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W50" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="W50" s="4" t="s">
+      <c r="X50" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X50" s="4" t="s">
+      <c r="Y50" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y50" s="5" t="s">
+      <c r="Z50" s="5" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="51" spans="1:25" ht="51.95" customHeight="1">
+    <row r="51" spans="1:26" ht="51.95" customHeight="1">
       <c r="A51" s="39" t="s">
         <v>57</v>
       </c>
@@ -7101,28 +7204,29 @@
       <c r="Q51" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R51" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S51" s="4"/>
+      <c r="R51" s="4"/>
+      <c r="S51" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T51" s="4"/>
-      <c r="U51" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U51" s="4"/>
       <c r="V51" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W51" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="W51" s="4" t="s">
+      <c r="X51" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X51" s="4" t="s">
+      <c r="Y51" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y51" s="5" t="s">
+      <c r="Z51" s="5" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="52" spans="1:25" ht="51.95" customHeight="1">
+    <row r="52" spans="1:26" ht="51.95" customHeight="1">
       <c r="A52" s="39" t="s">
         <v>57</v>
       </c>
@@ -7172,28 +7276,29 @@
       <c r="Q52" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R52" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S52" s="4"/>
+      <c r="R52" s="4"/>
+      <c r="S52" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T52" s="4"/>
-      <c r="U52" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U52" s="4"/>
       <c r="V52" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W52" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="W52" s="4" t="s">
+      <c r="X52" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X52" s="4" t="s">
+      <c r="Y52" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y52" s="5" t="s">
+      <c r="Z52" s="5" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="53" spans="1:25" ht="51.95" customHeight="1">
+    <row r="53" spans="1:26" ht="51.95" customHeight="1">
       <c r="A53" s="39" t="s">
         <v>57</v>
       </c>
@@ -7245,28 +7350,29 @@
       <c r="Q53" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R53" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S53" s="4"/>
+      <c r="R53" s="4"/>
+      <c r="S53" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T53" s="4"/>
-      <c r="U53" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U53" s="4"/>
       <c r="V53" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W53" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="W53" s="4" t="s">
+      <c r="X53" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X53" s="4" t="s">
+      <c r="Y53" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y53" s="5" t="s">
+      <c r="Z53" s="5" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="54" spans="1:25" ht="51.95" customHeight="1">
+    <row r="54" spans="1:26" ht="51.95" customHeight="1">
       <c r="A54" s="39" t="s">
         <v>57</v>
       </c>
@@ -7318,28 +7424,29 @@
       <c r="Q54" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R54" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S54" s="4"/>
+      <c r="R54" s="4"/>
+      <c r="S54" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T54" s="4"/>
-      <c r="U54" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U54" s="4"/>
       <c r="V54" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W54" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="W54" s="4" t="s">
+      <c r="X54" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X54" s="4" t="s">
+      <c r="Y54" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y54" s="5" t="s">
+      <c r="Z54" s="5" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="55" spans="1:25" ht="51.95" customHeight="1">
+    <row r="55" spans="1:26" ht="51.95" customHeight="1">
       <c r="A55" s="39" t="s">
         <v>57</v>
       </c>
@@ -7389,28 +7496,29 @@
       <c r="Q55" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R55" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S55" s="4"/>
+      <c r="R55" s="4"/>
+      <c r="S55" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T55" s="4"/>
-      <c r="U55" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U55" s="4"/>
       <c r="V55" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W55" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="W55" s="4" t="s">
+      <c r="X55" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X55" s="4" t="s">
+      <c r="Y55" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y55" s="5" t="s">
+      <c r="Z55" s="5" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="56" spans="1:25" ht="51.95" customHeight="1">
+    <row r="56" spans="1:26" ht="51.95" customHeight="1">
       <c r="A56" s="39" t="s">
         <v>57</v>
       </c>
@@ -7462,28 +7570,29 @@
       <c r="Q56" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R56" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S56" s="4"/>
+      <c r="R56" s="4"/>
+      <c r="S56" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T56" s="4"/>
-      <c r="U56" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U56" s="4"/>
       <c r="V56" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W56" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="W56" s="4" t="s">
+      <c r="X56" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X56" s="4" t="s">
+      <c r="Y56" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y56" s="5" t="s">
+      <c r="Z56" s="5" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="57" spans="1:25" ht="51.95" customHeight="1">
+    <row r="57" spans="1:26" ht="51.95" customHeight="1">
       <c r="A57" s="39" t="s">
         <v>57</v>
       </c>
@@ -7533,28 +7642,29 @@
       <c r="Q57" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R57" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S57" s="4"/>
+      <c r="R57" s="4"/>
+      <c r="S57" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T57" s="4"/>
-      <c r="U57" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U57" s="4"/>
       <c r="V57" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W57" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="W57" s="4" t="s">
+      <c r="X57" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X57" s="4" t="s">
+      <c r="Y57" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y57" s="5" t="s">
+      <c r="Z57" s="5" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="58" spans="1:25" ht="51.95" customHeight="1">
+    <row r="58" spans="1:26" ht="51.95" customHeight="1">
       <c r="A58" s="39" t="s">
         <v>57</v>
       </c>
@@ -7606,28 +7716,29 @@
       <c r="Q58" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R58" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S58" s="4"/>
+      <c r="R58" s="4"/>
+      <c r="S58" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T58" s="4"/>
-      <c r="U58" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U58" s="4"/>
       <c r="V58" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W58" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="W58" s="4" t="s">
+      <c r="X58" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X58" s="4" t="s">
+      <c r="Y58" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y58" s="5" t="s">
+      <c r="Z58" s="5" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="59" spans="1:25" ht="51.95" customHeight="1">
+    <row r="59" spans="1:26" ht="51.95" customHeight="1">
       <c r="A59" s="39" t="s">
         <v>57</v>
       </c>
@@ -7679,28 +7790,29 @@
       <c r="Q59" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R59" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S59" s="4"/>
+      <c r="R59" s="4"/>
+      <c r="S59" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="T59" s="4"/>
-      <c r="U59" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="U59" s="4"/>
       <c r="V59" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="W59" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="W59" s="4" t="s">
+      <c r="X59" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X59" s="4" t="s">
+      <c r="Y59" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="Y59" s="5" t="s">
+      <c r="Z59" s="5" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="60" spans="1:25" ht="51.95" customHeight="1">
+    <row r="60" spans="1:26" ht="51.95" customHeight="1">
       <c r="A60" s="39" t="s">
         <v>57</v>
       </c>
@@ -7748,54 +7860,55 @@
       <c r="Q60" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="R60" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="S60" s="6"/>
+      <c r="R60" s="6"/>
+      <c r="S60" s="6" t="s">
+        <v>57</v>
+      </c>
       <c r="T60" s="6"/>
-      <c r="U60" s="6" t="s">
-        <v>57</v>
-      </c>
+      <c r="U60" s="6"/>
       <c r="V60" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="W60" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="W60" s="6" t="s">
+      <c r="X60" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="X60" s="6" t="s">
+      <c r="Y60" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="Y60" s="7" t="s">
+      <c r="Z60" s="7" t="s">
         <v>283</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B1:Y1"/>
-    <mergeCell ref="B2:Y2"/>
+    <mergeCell ref="B1:Z1"/>
+    <mergeCell ref="B2:Z2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:Y27 A29:O29 Q28:Y29 A28:N28 A30:Y33 A34:O34 Q34:Y34 A35:Y60">
+  <conditionalFormatting sqref="A28:N28 Q28:Z29 A29:O29 A30:Z33 A34:O34 Q34:Z34 A5:Z27 A35:Z60">
     <cfRule type="expression" dxfId="4" priority="3">
       <formula>$E5="Must"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W5:W60">
-    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="Pending"/>
+  <conditionalFormatting sqref="O28:P28">
+    <cfRule type="expression" dxfId="3" priority="2">
+      <formula>$E28="Must"</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P29">
     <cfRule type="expression" dxfId="2" priority="8">
       <formula>$E28="Must"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O28:P28">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>$E28="Must"</formula>
+  <conditionalFormatting sqref="P34">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>$E34="Must"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P34">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>$E34="Must"</formula>
-    </cfRule>
+  <conditionalFormatting sqref="X5:X60">
+    <cfRule type="containsText" dxfId="0" priority="6" operator="containsText" text="Pending"/>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" sqref="B5:B60" xr:uid="{00000000-0002-0000-0100-000000000000}">

</xml_diff>

<commit_message>
BRD and RTM updates along with docs relating to twitter posts
</commit_message>
<xml_diff>
--- a/docs/project-management/02_Business_Requirements/Northwind-Outdoor-RTM-v1.0.xlsx
+++ b/docs/project-management/02_Business_Requirements/Northwind-Outdoor-RTM-v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/docs/project-management/02_Business_Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="784" documentId="8_{170D4D7C-E242-4887-90C6-7A678B36976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30CC72D7-AC51-4E30-8460-6C0F686F2BF5}"/>
+  <xr:revisionPtr revIDLastSave="785" documentId="8_{170D4D7C-E242-4887-90C6-7A678B36976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19A492DE-21E7-4B61-BCAA-22328CBB8AEE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3207,10 +3207,10 @@
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="HLD (Primary)"/>
     <tableColumn id="24" xr3:uid="{599BD185-8391-4930-BB9A-B52E39596ACD}" name="HLD (Secondary)" dataDxfId="8"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="LLD (Primary)"/>
-    <tableColumn id="10" xr3:uid="{D9149C79-EC24-41C1-B36D-CD2D9225FFA3}" name="LLD (Secondary)" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{D9149C79-EC24-41C1-B36D-CD2D9225FFA3}" name="LLD (Secondary)" dataDxfId="7"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="ADR"/>
-    <tableColumn id="25" xr3:uid="{28378BB4-B208-482C-96C2-5A1994DECC42}" name="SOW" dataDxfId="7"/>
-    <tableColumn id="26" xr3:uid="{BAEC8EC4-D90B-4FBA-979D-21CDBE3C330A}" name="Sprint" dataDxfId="6"/>
+    <tableColumn id="25" xr3:uid="{28378BB4-B208-482C-96C2-5A1994DECC42}" name="SOW" dataDxfId="6"/>
+    <tableColumn id="26" xr3:uid="{BAEC8EC4-D90B-4FBA-979D-21CDBE3C330A}" name="Sprint" dataDxfId="5"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Test / UAT"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Acceptance Criteria"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Status"/>
@@ -3645,7 +3645,7 @@
   <dimension ref="A1:Z60"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.625" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="13.375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
@@ -7887,7 +7887,7 @@
     <mergeCell ref="B1:Z1"/>
     <mergeCell ref="B2:Z2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A28:N28 Q28:Z29 A29:O29 A30:Z33 A34:O34 Q34:Z34 A5:Z27 A35:Z60">
+  <conditionalFormatting sqref="A5:Z27 A28:N28 Q28:Z29 A29:O29 A30:Z33 A34:O34 Q34:Z34 A35:Z60">
     <cfRule type="expression" dxfId="4" priority="3">
       <formula>$E5="Must"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Initial draft HYP01 documentation
</commit_message>
<xml_diff>
--- a/docs/project-management/02_Business_Requirements/Northwind-Outdoor-RTM-v1.0.xlsx
+++ b/docs/project-management/02_Business_Requirements/Northwind-Outdoor-RTM-v1.0.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/docs/project-management/02_Business_Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="785" documentId="8_{170D4D7C-E242-4887-90C6-7A678B36976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19A492DE-21E7-4B61-BCAA-22328CBB8AEE}"/>
+  <xr:revisionPtr revIDLastSave="789" documentId="8_{170D4D7C-E242-4887-90C6-7A678B36976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C381DF28-FFE1-4755-8D2F-0EF22ED441F8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>